<commit_message>
Corrected NetApp status to Target Selected for Applied Queue
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -5247,7 +5247,7 @@
       </c>
       <c r="H71" s="20" t="inlineStr">
         <is>
-          <t>Submitted / Target Applied</t>
+          <t>Reviewed - Target Selected for Applied Queue</t>
         </is>
       </c>
       <c r="I71" s="20" t="inlineStr">
@@ -5277,7 +5277,7 @@
       </c>
       <c r="N71" s="20" t="inlineStr">
         <is>
-          <t>NetApp Bangalore hybrid opening for Business Analyst. 95% skill match (Power BI, SQL, Data Quality, Automated Scorecards, EDW). Requirement asks min 4+ Yrs exp.</t>
+          <t>Target role selected from NetApp Workday careers portal for Business Analyst (Data &amp; Finance Analytics). Pending direct web form submission.</t>
         </is>
       </c>
       <c r="O71" s="20" t="inlineStr">

</xml_diff>

<commit_message>
Logged Ankit Kumar (VP at Pyramid IT Consulting) NVite outreach
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -702,7 +702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O94"/>
+  <dimension ref="A1:O95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="17" min="1" max="1"/>
@@ -6775,7 +6775,81 @@
         </is>
       </c>
     </row>
-    <row r="95" ht="33.95" customHeight="1" s="17"/>
+    <row r="95" ht="33.95" customHeight="1" s="17">
+      <c r="A95" s="20" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B95" s="20" t="inlineStr">
+        <is>
+          <t>Pyramid IT Consulting</t>
+        </is>
+      </c>
+      <c r="C95" s="20" t="inlineStr">
+        <is>
+          <t>Senior Data / IT Role (Naukri NVite)</t>
+        </is>
+      </c>
+      <c r="D95" s="20" t="inlineStr">
+        <is>
+          <t>NOIDA / Remote</t>
+        </is>
+      </c>
+      <c r="E95" s="20" t="inlineStr">
+        <is>
+          <t>Naukri Recruiter Direct NVite</t>
+        </is>
+      </c>
+      <c r="F95" s="20" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G95" s="20" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H95" s="20" t="inlineStr">
+        <is>
+          <t>NVite Received (Accepted &amp; Profile Connected)</t>
+        </is>
+      </c>
+      <c r="I95" s="20" t="inlineStr">
+        <is>
+          <t>Ankit Kumar (VP at Pyramid IT Consulting)</t>
+        </is>
+      </c>
+      <c r="J95" s="20" t="inlineStr">
+        <is>
+          <t>Noida Direct NVite</t>
+        </is>
+      </c>
+      <c r="K95" s="20" t="inlineStr">
+        <is>
+          <t>NVite received from VP level recruiter (Ankit Kumar, VP at Pyramid IT Consulting). NVite accepted on Naukri.</t>
+        </is>
+      </c>
+      <c r="L95" s="20" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="M95" s="20" t="inlineStr">
+        <is>
+          <t>Not Disclosed / Senior CTC Band</t>
+        </is>
+      </c>
+      <c r="N95" s="20" t="inlineStr">
+        <is>
+          <t>VP level outreach from Pyramid IT Consulting (Ankit Kumar, VP). NVite accepted on Naukri.</t>
+        </is>
+      </c>
+      <c r="O95" s="20" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
     <row r="96" ht="33.95" customHeight="1" s="17"/>
     <row r="97" ht="33.95" customHeight="1" s="17"/>
     <row r="98" ht="33.95" customHeight="1" s="17"/>

</xml_diff>

<commit_message>
Tuesday Aug 11: Logged 2 Growel Softech Snowflake NVites (Row 96 & 97) submitted on Naukri
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Carlito"/>
       <sz val="11"/>
@@ -75,8 +75,12 @@
       <color rgb="FF4B5563"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Carlito"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -141,20 +145,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-        <bgColor rgb="00C6EFCE"/>
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-        <bgColor rgb="00FFC7CE"/>
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor rgb="FFFFC7CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
-        <bgColor rgb="00FFF2CC"/>
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -212,10 +222,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="2">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -243,13 +254,18 @@
     <xf numFmtId="0" fontId="9" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="11" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -262,17 +278,21 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="9" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="9" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="9" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="12">
     <dxf>
@@ -488,7 +508,7 @@
     <tableColumn id="3" name="Role"/>
     <tableColumn id="4" name="Location"/>
     <tableColumn id="5" name="Source"/>
-    <tableColumn id="6" name="Match %"/>
+    <tableColumn id="6" name="Match %" dataCellStyle="Percent"/>
     <tableColumn id="7" name="Resume Version"/>
     <tableColumn id="8" name="Application Status"/>
     <tableColumn id="9" name="Recruiter Name"/>
@@ -702,41 +722,41 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O95"/>
+  <dimension ref="A1:O97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
-    <col width="13" customWidth="1" style="17" min="1" max="1"/>
-    <col width="29.25" bestFit="1" customWidth="1" style="17" min="2" max="2"/>
-    <col width="22" customWidth="1" style="17" min="3" max="3"/>
-    <col width="16" customWidth="1" style="17" min="4" max="4"/>
-    <col width="14" customWidth="1" style="17" min="5" max="5"/>
-    <col width="10" customWidth="1" style="17" min="6" max="6"/>
-    <col width="30" customWidth="1" style="17" min="7" max="7"/>
-    <col width="26.375" bestFit="1" customWidth="1" style="17" min="8" max="8"/>
-    <col width="20" customWidth="1" style="17" min="9" max="9"/>
-    <col width="25" customWidth="1" style="17" min="10" max="10"/>
-    <col width="22" customWidth="1" style="17" min="11" max="11"/>
-    <col width="14" customWidth="1" style="17" min="12" max="12"/>
-    <col width="20" customWidth="1" style="17" min="13" max="13"/>
-    <col width="32" customWidth="1" style="17" min="14" max="14"/>
-    <col width="16" customWidth="1" style="17" min="15" max="15"/>
+    <col width="13" customWidth="1" style="20" min="1" max="1"/>
+    <col width="29.25" bestFit="1" customWidth="1" style="20" min="2" max="2"/>
+    <col width="22" customWidth="1" style="20" min="3" max="3"/>
+    <col width="16" customWidth="1" style="20" min="4" max="4"/>
+    <col width="14" customWidth="1" style="20" min="5" max="5"/>
+    <col width="10" customWidth="1" style="28" min="6" max="6"/>
+    <col width="30" customWidth="1" style="20" min="7" max="7"/>
+    <col width="26.375" bestFit="1" customWidth="1" style="20" min="8" max="8"/>
+    <col width="20" customWidth="1" style="20" min="9" max="9"/>
+    <col width="25" customWidth="1" style="20" min="10" max="10"/>
+    <col width="22" customWidth="1" style="20" min="11" max="11"/>
+    <col width="14" customWidth="1" style="20" min="12" max="12"/>
+    <col width="20" customWidth="1" style="20" min="13" max="13"/>
+    <col width="32" customWidth="1" style="20" min="14" max="14"/>
+    <col width="16" customWidth="1" style="20" min="15" max="15"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" s="17">
-      <c r="A1" s="16" t="inlineStr">
+    <row r="1" ht="30" customHeight="1" s="20">
+      <c r="A1" s="19" t="inlineStr">
         <is>
           <t>Job Application Tracker</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="24" customHeight="1" s="17">
-      <c r="A2" s="18" t="inlineStr">
+    <row r="2" ht="24" customHeight="1" s="20">
+      <c r="A2" s="21" t="inlineStr">
         <is>
           <t>Track applications, interviews, follow-ups, and outcomes. Update the Status and Follow-up Date after every action.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="32.1" customHeight="1" s="17">
+    <row r="4" ht="32.1" customHeight="1" s="20">
       <c r="A4" s="1" t="inlineStr">
         <is>
           <t>Date Applied</t>
@@ -762,7 +782,7 @@
           <t>Source</t>
         </is>
       </c>
-      <c r="F4" s="1" t="inlineStr">
+      <c r="F4" s="23" t="inlineStr">
         <is>
           <t>Match %</t>
         </is>
@@ -813,7 +833,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="21.95" customHeight="1" s="17">
+    <row r="5" ht="21.95" customHeight="1" s="20">
       <c r="A5" s="6" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -839,7 +859,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F5" s="6" t="n">
+      <c r="F5" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -847,7 +867,7 @@
           <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
         </is>
       </c>
-      <c r="H5" s="22" t="inlineStr">
+      <c r="H5" s="17" t="inlineStr">
         <is>
           <t>L1 Senior Technical Interview Completed &amp; Rated (Risebird)</t>
         </is>
@@ -888,7 +908,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="21.95" customHeight="1" s="17">
+    <row r="6" ht="21.95" customHeight="1" s="20">
       <c r="A6" s="6" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -914,7 +934,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F6" s="6" t="n">
+      <c r="F6" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -951,7 +971,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="21.95" customHeight="1" s="17">
+    <row r="7" ht="21.95" customHeight="1" s="20">
       <c r="A7" s="6" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -977,7 +997,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F7" s="6" t="n">
+      <c r="F7" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -985,7 +1005,7 @@
           <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
         </is>
       </c>
-      <c r="H7" s="15" t="inlineStr">
+      <c r="H7" s="13" t="inlineStr">
         <is>
           <t>Referral Confirmation Received</t>
         </is>
@@ -1026,7 +1046,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="21.95" customHeight="1" s="17">
+    <row r="8" ht="21.95" customHeight="1" s="20">
       <c r="A8" s="6" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -1052,7 +1072,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F8" s="6" t="n">
+      <c r="F8" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -1093,7 +1113,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="21.95" customHeight="1" s="17">
+    <row r="9" ht="21.95" customHeight="1" s="20">
       <c r="A9" s="6" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -1119,7 +1139,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F9" s="6" t="n">
+      <c r="F9" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -1156,7 +1176,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="21.95" customHeight="1" s="17">
+    <row r="10" ht="21.95" customHeight="1" s="20">
       <c r="A10" s="6" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -1182,7 +1202,7 @@
           <t>Naukri</t>
         </is>
       </c>
-      <c r="F10" s="6" t="n">
+      <c r="F10" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -1219,7 +1239,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="21.95" customHeight="1" s="17">
+    <row r="11" ht="21.95" customHeight="1" s="20">
       <c r="A11" s="6" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -1245,7 +1265,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F11" s="6" t="n">
+      <c r="F11" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -1286,7 +1306,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="21.95" customHeight="1" s="17">
+    <row r="12" ht="21.95" customHeight="1" s="20">
       <c r="A12" s="6" t="inlineStr">
         <is>
           <t>2026-08-01</t>
@@ -1312,7 +1332,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F12" s="6" t="n">
+      <c r="F12" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G12" s="7" t="inlineStr">
@@ -1349,7 +1369,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="21.95" customHeight="1" s="17">
+    <row r="13" ht="21.95" customHeight="1" s="20">
       <c r="A13" s="6" t="inlineStr">
         <is>
           <t>2026-08-01</t>
@@ -1375,7 +1395,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F13" s="6" t="n">
+      <c r="F13" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -1412,7 +1432,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="21.95" customHeight="1" s="17">
+    <row r="14" ht="21.95" customHeight="1" s="20">
       <c r="A14" s="6" t="inlineStr">
         <is>
           <t>2026-08-01</t>
@@ -1438,7 +1458,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F14" s="6" t="n">
+      <c r="F14" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G14" s="7" t="inlineStr">
@@ -1475,7 +1495,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="21.95" customHeight="1" s="17">
+    <row r="15" ht="21.95" customHeight="1" s="20">
       <c r="A15" s="6" t="inlineStr">
         <is>
           <t>2026-08-01</t>
@@ -1501,7 +1521,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F15" s="6" t="n">
+      <c r="F15" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -1538,7 +1558,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="21.95" customHeight="1" s="17">
+    <row r="16" ht="21.95" customHeight="1" s="20">
       <c r="A16" s="6" t="inlineStr">
         <is>
           <t>2026-08-01</t>
@@ -1564,7 +1584,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F16" s="6" t="n">
+      <c r="F16" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G16" s="7" t="inlineStr">
@@ -1605,7 +1625,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="21.95" customHeight="1" s="17">
+    <row r="17" ht="21.95" customHeight="1" s="20">
       <c r="A17" s="6" t="inlineStr">
         <is>
           <t>2026-07-31</t>
@@ -1631,7 +1651,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F17" s="6" t="n">
+      <c r="F17" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G17" s="7" t="inlineStr">
@@ -1672,7 +1692,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="21.95" customHeight="1" s="17">
+    <row r="18" ht="21.95" customHeight="1" s="20">
       <c r="A18" s="6" t="inlineStr">
         <is>
           <t>2026-07-31</t>
@@ -1698,7 +1718,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F18" s="6" t="n">
+      <c r="F18" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G18" s="7" t="inlineStr">
@@ -1735,7 +1755,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="21.95" customHeight="1" s="17">
+    <row r="19" ht="21.95" customHeight="1" s="20">
       <c r="A19" s="6" t="inlineStr">
         <is>
           <t>2026-07-31</t>
@@ -1761,7 +1781,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F19" s="6" t="n">
+      <c r="F19" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -1802,7 +1822,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="21.95" customHeight="1" s="17">
+    <row r="20" ht="21.95" customHeight="1" s="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
           <t>2026-07-31</t>
@@ -1828,7 +1848,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F20" s="6" t="n">
+      <c r="F20" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G20" s="7" t="inlineStr">
@@ -1836,9 +1856,9 @@
           <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
         </is>
       </c>
-      <c r="H20" s="23" t="inlineStr">
-        <is>
-          <t>CAUTION: Deputated Staffing Payroll Risk (AmbitionBox 2.8/5 Rating)</t>
+      <c r="H20" s="18" t="inlineStr">
+        <is>
+          <t>Awaiting Calendar Slot Confirmation (Persistent Systems Stage 2)</t>
         </is>
       </c>
       <c r="I20" s="7" t="inlineStr">
@@ -1868,7 +1888,7 @@
       </c>
       <c r="N20" s="7" t="inlineStr">
         <is>
-          <t>AmbitionBox Audit: Growel Softech has 2.8/5 rating. Issues: Salary delays, HR ghosting, third-party payroll agency for Persistent Systems. Strategy: Prioritize direct enterprise payrolls (Mphasis, Wells Fargo, Euronext, Nisvan 22.5-25 LPA).</t>
+          <t>Pooja (Growel Softech) confirmed candidate shortlisted for Stage 2 Human Technical Round. Awaiting calendar invite/slot confirmation call from Persistent Systems.</t>
         </is>
       </c>
       <c r="O20" s="6" t="inlineStr">
@@ -1877,7 +1897,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="21.95" customHeight="1" s="17">
+    <row r="21" ht="21.95" customHeight="1" s="20">
       <c r="A21" s="6" t="inlineStr">
         <is>
           <t>2026-07-31</t>
@@ -1903,7 +1923,7 @@
           <t>Naukri</t>
         </is>
       </c>
-      <c r="F21" s="6" t="n">
+      <c r="F21" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G21" s="7" t="inlineStr">
@@ -1940,7 +1960,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="21.95" customHeight="1" s="17">
+    <row r="22" ht="21.95" customHeight="1" s="20">
       <c r="A22" s="6" t="inlineStr">
         <is>
           <t>2026-07-31</t>
@@ -1966,7 +1986,7 @@
           <t>Naukri</t>
         </is>
       </c>
-      <c r="F22" s="6" t="n">
+      <c r="F22" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G22" s="7" t="inlineStr">
@@ -2003,7 +2023,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="21.95" customHeight="1" s="17">
+    <row r="23" ht="21.95" customHeight="1" s="20">
       <c r="A23" s="6" t="inlineStr">
         <is>
           <t>2026-07-31</t>
@@ -2029,7 +2049,7 @@
           <t>Naukri</t>
         </is>
       </c>
-      <c r="F23" s="6" t="n">
+      <c r="F23" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G23" s="7" t="inlineStr">
@@ -2066,7 +2086,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="21.95" customHeight="1" s="17">
+    <row r="24" ht="21.95" customHeight="1" s="20">
       <c r="A24" s="6" t="inlineStr">
         <is>
           <t>2026-07-31</t>
@@ -2092,7 +2112,7 @@
           <t>Naukri</t>
         </is>
       </c>
-      <c r="F24" s="6" t="n">
+      <c r="F24" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G24" s="7" t="inlineStr">
@@ -2129,7 +2149,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="21.95" customHeight="1" s="17">
+    <row r="25" ht="21.95" customHeight="1" s="20">
       <c r="A25" s="6" t="inlineStr">
         <is>
           <t>2026-07-31</t>
@@ -2155,7 +2175,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F25" s="6" t="n">
+      <c r="F25" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G25" s="7" t="inlineStr">
@@ -2192,7 +2212,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="21.95" customHeight="1" s="17">
+    <row r="26" ht="21.95" customHeight="1" s="20">
       <c r="A26" s="6" t="inlineStr">
         <is>
           <t>2026-07-31</t>
@@ -2218,7 +2238,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F26" s="6" t="n">
+      <c r="F26" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G26" s="7" t="inlineStr">
@@ -2255,7 +2275,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="21.95" customHeight="1" s="17">
+    <row r="27" ht="21.95" customHeight="1" s="20">
       <c r="A27" s="6" t="inlineStr">
         <is>
           <t>2026-07-31</t>
@@ -2281,7 +2301,7 @@
           <t>Naukri</t>
         </is>
       </c>
-      <c r="F27" s="6" t="n">
+      <c r="F27" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G27" s="7" t="inlineStr">
@@ -2322,7 +2342,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="21.95" customHeight="1" s="17">
+    <row r="28" ht="21.95" customHeight="1" s="20">
       <c r="A28" s="6" t="inlineStr">
         <is>
           <t>2026-07-29</t>
@@ -2348,7 +2368,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F28" s="6" t="n">
+      <c r="F28" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G28" s="7" t="inlineStr">
@@ -2385,7 +2405,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="21.95" customHeight="1" s="17">
+    <row r="29" ht="21.95" customHeight="1" s="20">
       <c r="A29" s="6" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -2411,7 +2431,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F29" s="6" t="n">
+      <c r="F29" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G29" s="7" t="inlineStr">
@@ -2448,7 +2468,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="21.95" customHeight="1" s="17">
+    <row r="30" ht="21.95" customHeight="1" s="20">
       <c r="A30" s="6" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -2474,7 +2494,7 @@
           <t>Naukri</t>
         </is>
       </c>
-      <c r="F30" s="6" t="n">
+      <c r="F30" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G30" s="7" t="inlineStr">
@@ -2519,7 +2539,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="21.95" customHeight="1" s="17">
+    <row r="31" ht="21.95" customHeight="1" s="20">
       <c r="A31" s="6" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -2545,7 +2565,7 @@
           <t>Naukri</t>
         </is>
       </c>
-      <c r="F31" s="6" t="n">
+      <c r="F31" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G31" s="7" t="inlineStr">
@@ -2582,7 +2602,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="21.95" customHeight="1" s="17">
+    <row r="32" ht="21.95" customHeight="1" s="20">
       <c r="A32" s="6" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -2608,7 +2628,7 @@
           <t>Naukri</t>
         </is>
       </c>
-      <c r="F32" s="6" t="n">
+      <c r="F32" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G32" s="7" t="inlineStr">
@@ -2645,7 +2665,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="21.95" customHeight="1" s="17">
+    <row r="33" ht="21.95" customHeight="1" s="20">
       <c r="A33" s="6" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -2671,7 +2691,7 @@
           <t>Wellfound</t>
         </is>
       </c>
-      <c r="F33" s="6" t="n">
+      <c r="F33" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G33" s="7" t="inlineStr">
@@ -2708,7 +2728,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="21.95" customHeight="1" s="17">
+    <row r="34" ht="21.95" customHeight="1" s="20">
       <c r="A34" s="6" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -2734,7 +2754,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F34" s="6" t="n">
+      <c r="F34" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G34" s="7" t="inlineStr">
@@ -2775,7 +2795,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="21.95" customHeight="1" s="17">
+    <row r="35" ht="21.95" customHeight="1" s="20">
       <c r="A35" s="6" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -2801,7 +2821,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F35" s="6" t="n">
+      <c r="F35" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G35" s="7" t="inlineStr">
@@ -2838,7 +2858,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="21.95" customHeight="1" s="17">
+    <row r="36" ht="21.95" customHeight="1" s="20">
       <c r="A36" s="6" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -2864,7 +2884,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F36" s="6" t="n">
+      <c r="F36" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G36" s="7" t="inlineStr">
@@ -2901,7 +2921,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="21.95" customHeight="1" s="17">
+    <row r="37" ht="21.95" customHeight="1" s="20">
       <c r="A37" s="6" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -2927,7 +2947,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F37" s="6" t="n">
+      <c r="F37" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G37" s="7" t="inlineStr">
@@ -2964,7 +2984,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="21.95" customHeight="1" s="17">
+    <row r="38" ht="21.95" customHeight="1" s="20">
       <c r="A38" s="6" t="inlineStr">
         <is>
           <t>2026-07-28</t>
@@ -2990,7 +3010,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F38" s="6" t="n">
+      <c r="F38" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G38" s="7" t="inlineStr">
@@ -3027,7 +3047,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="21.95" customHeight="1" s="17">
+    <row r="39" ht="21.95" customHeight="1" s="20">
       <c r="A39" s="6" t="inlineStr">
         <is>
           <t>2026-07-27</t>
@@ -3053,7 +3073,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F39" s="6" t="n">
+      <c r="F39" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G39" s="7" t="inlineStr">
@@ -3094,7 +3114,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="21.95" customHeight="1" s="17">
+    <row r="40" ht="21.95" customHeight="1" s="20">
       <c r="A40" s="6" t="inlineStr">
         <is>
           <t>2026-07-27</t>
@@ -3120,7 +3140,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F40" s="6" t="n">
+      <c r="F40" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G40" s="7" t="inlineStr">
@@ -3161,7 +3181,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="21.95" customHeight="1" s="17">
+    <row r="41" ht="21.95" customHeight="1" s="20">
       <c r="A41" s="6" t="inlineStr">
         <is>
           <t>2026-07-27</t>
@@ -3187,7 +3207,7 @@
           <t>Company Portal</t>
         </is>
       </c>
-      <c r="F41" s="6" t="n">
+      <c r="F41" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G41" s="7" t="inlineStr">
@@ -3224,7 +3244,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="21.95" customHeight="1" s="17">
+    <row r="42" ht="21.95" customHeight="1" s="20">
       <c r="A42" s="6" t="inlineStr">
         <is>
           <t>2026-07-27</t>
@@ -3250,7 +3270,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F42" s="6" t="n">
+      <c r="F42" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G42" s="7" t="inlineStr">
@@ -3287,7 +3307,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="21.95" customHeight="1" s="17">
+    <row r="43" ht="21.95" customHeight="1" s="20">
       <c r="A43" s="6" t="inlineStr">
         <is>
           <t>2026-07-27</t>
@@ -3313,7 +3333,7 @@
           <t>Naukri</t>
         </is>
       </c>
-      <c r="F43" s="6" t="n">
+      <c r="F43" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G43" s="7" t="inlineStr">
@@ -3350,7 +3370,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="21.95" customHeight="1" s="17">
+    <row r="44" ht="21.95" customHeight="1" s="20">
       <c r="A44" s="6" t="inlineStr">
         <is>
           <t>2026-07-27</t>
@@ -3376,7 +3396,7 @@
           <t>Company Portal</t>
         </is>
       </c>
-      <c r="F44" s="6" t="n">
+      <c r="F44" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G44" s="7" t="inlineStr">
@@ -3413,7 +3433,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="21.95" customHeight="1" s="17">
+    <row r="45" ht="21.95" customHeight="1" s="20">
       <c r="A45" s="6" t="inlineStr">
         <is>
           <t>2026-08-07</t>
@@ -3439,7 +3459,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F45" s="6" t="n">
+      <c r="F45" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G45" s="7" t="inlineStr">
@@ -3447,7 +3467,7 @@
           <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
         </is>
       </c>
-      <c r="H45" s="22" t="inlineStr">
+      <c r="H45" s="17" t="inlineStr">
         <is>
           <t>Application Re-Submitted via LinkedIn Easy Apply</t>
         </is>
@@ -3476,7 +3496,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="21.95" customHeight="1" s="17">
+    <row r="46" ht="21.95" customHeight="1" s="20">
       <c r="A46" s="6" t="inlineStr">
         <is>
           <t>2026-07-27</t>
@@ -3502,7 +3522,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F46" s="6" t="n">
+      <c r="F46" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G46" s="7" t="inlineStr">
@@ -3543,7 +3563,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="21.95" customHeight="1" s="17">
+    <row r="47" ht="21.95" customHeight="1" s="20">
       <c r="A47" s="6" t="inlineStr">
         <is>
           <t>2026-07-27</t>
@@ -3569,7 +3589,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F47" s="6" t="n">
+      <c r="F47" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G47" s="7" t="inlineStr">
@@ -3606,7 +3626,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="21.95" customHeight="1" s="17">
+    <row r="48" ht="21.95" customHeight="1" s="20">
       <c r="A48" s="6" t="inlineStr">
         <is>
           <t>2026-07-27</t>
@@ -3632,7 +3652,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F48" s="6" t="n">
+      <c r="F48" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G48" s="7" t="inlineStr">
@@ -3673,7 +3693,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="21.95" customHeight="1" s="17">
+    <row r="49" ht="21.95" customHeight="1" s="20">
       <c r="A49" s="6" t="inlineStr">
         <is>
           <t>2026-07-27</t>
@@ -3699,7 +3719,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F49" s="6" t="n">
+      <c r="F49" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G49" s="7" t="inlineStr">
@@ -3740,7 +3760,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="21.95" customHeight="1" s="17">
+    <row r="50" ht="21.95" customHeight="1" s="20">
       <c r="A50" s="6" t="inlineStr">
         <is>
           <t>2026-07-27</t>
@@ -3766,7 +3786,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F50" s="6" t="n">
+      <c r="F50" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G50" s="7" t="inlineStr">
@@ -3803,7 +3823,7 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="21.95" customHeight="1" s="17">
+    <row r="51" ht="21.95" customHeight="1" s="20">
       <c r="A51" s="6" t="inlineStr">
         <is>
           <t>2026-07-27</t>
@@ -3829,7 +3849,7 @@
           <t>Wellfound</t>
         </is>
       </c>
-      <c r="F51" s="6" t="n">
+      <c r="F51" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G51" s="7" t="inlineStr">
@@ -3870,7 +3890,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="21.95" customHeight="1" s="17">
+    <row r="52" ht="21.95" customHeight="1" s="20">
       <c r="A52" s="6" t="inlineStr">
         <is>
           <t>2026-07-27</t>
@@ -3896,7 +3916,7 @@
           <t>Wellfound</t>
         </is>
       </c>
-      <c r="F52" s="6" t="n">
+      <c r="F52" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G52" s="7" t="inlineStr">
@@ -3937,7 +3957,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="21.95" customHeight="1" s="17">
+    <row r="53" ht="21.95" customHeight="1" s="20">
       <c r="A53" s="6" t="inlineStr">
         <is>
           <t>2026-07-27</t>
@@ -3963,7 +3983,7 @@
           <t>Wellfound</t>
         </is>
       </c>
-      <c r="F53" s="6" t="n">
+      <c r="F53" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G53" s="7" t="inlineStr">
@@ -4000,7 +4020,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="21.95" customHeight="1" s="17">
+    <row r="54" ht="21.95" customHeight="1" s="20">
       <c r="A54" s="6" t="inlineStr">
         <is>
           <t>2026-07-27</t>
@@ -4026,7 +4046,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F54" s="6" t="n">
+      <c r="F54" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G54" s="7" t="inlineStr">
@@ -4063,7 +4083,7 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="21.95" customHeight="1" s="17">
+    <row r="55" ht="21.95" customHeight="1" s="20">
       <c r="A55" s="6" t="inlineStr">
         <is>
           <t>2026-07-25</t>
@@ -4089,7 +4109,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F55" s="6" t="n">
+      <c r="F55" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G55" s="7" t="inlineStr">
@@ -4126,7 +4146,7 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="21.95" customHeight="1" s="17">
+    <row r="56" ht="21.95" customHeight="1" s="20">
       <c r="A56" s="6" t="inlineStr">
         <is>
           <t>2026-07-24</t>
@@ -4152,7 +4172,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F56" s="6" t="n">
+      <c r="F56" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G56" s="7" t="inlineStr">
@@ -4189,7 +4209,7 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="21.95" customHeight="1" s="17">
+    <row r="57" ht="21.95" customHeight="1" s="20">
       <c r="A57" s="6" t="inlineStr">
         <is>
           <t>2026-07-24</t>
@@ -4215,7 +4235,7 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F57" s="6" t="n">
+      <c r="F57" s="24" t="n">
         <v>0.9</v>
       </c>
       <c r="G57" s="7" t="inlineStr">
@@ -4252,591 +4272,591 @@
         </is>
       </c>
     </row>
-    <row r="58" ht="33.95" customHeight="1" s="17">
-      <c r="A58" s="13" t="inlineStr">
+    <row r="58" ht="33.95" customHeight="1" s="20">
+      <c r="A58" s="11" t="inlineStr">
         <is>
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="B58" s="13" t="inlineStr">
+      <c r="B58" s="11" t="inlineStr">
         <is>
           <t>Sigmoid</t>
         </is>
       </c>
-      <c r="C58" s="13" t="inlineStr">
+      <c r="C58" s="11" t="inlineStr">
         <is>
           <t>BI Solutions Architect</t>
         </is>
       </c>
-      <c r="D58" s="13" t="inlineStr">
+      <c r="D58" s="11" t="inlineStr">
         <is>
           <t>Bengaluru (Hybrid)</t>
         </is>
       </c>
-      <c r="E58" s="13" t="inlineStr">
+      <c r="E58" s="11" t="inlineStr">
         <is>
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="F58" s="13" t="n">
+      <c r="F58" s="25" t="n">
         <v>0.5</v>
       </c>
-      <c r="G58" s="13" t="inlineStr">
+      <c r="G58" s="11" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="H58" s="13" t="inlineStr">
+      <c r="H58" s="11" t="inlineStr">
         <is>
           <t>Not Applied - Skill Gap</t>
         </is>
       </c>
-      <c r="I58" s="13" t="inlineStr">
+      <c r="I58" s="11" t="inlineStr">
         <is>
           <t>Jeeba Tojo (Sr Lead TA)</t>
         </is>
       </c>
-      <c r="J58" s="13" t="inlineStr">
+      <c r="J58" s="11" t="inlineStr">
         <is>
           <t>LinkedIn DM</t>
         </is>
       </c>
-      <c r="K58" s="13" t="inlineStr">
+      <c r="K58" s="11" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="L58" s="13" t="n"/>
-      <c r="M58" s="13" t="inlineStr">
+      <c r="L58" s="11" t="n"/>
+      <c r="M58" s="11" t="inlineStr">
         <is>
           <t>Not Specified</t>
         </is>
       </c>
-      <c r="N58" s="13" t="inlineStr">
+      <c r="N58" s="11" t="inlineStr">
         <is>
           <t>JD reviewed. Major gaps: Tableau, React, Node.js, Docker, Databricks, Fabric APIs. Not a core match.</t>
         </is>
       </c>
-      <c r="O58" s="13" t="inlineStr">
+      <c r="O58" s="11" t="inlineStr">
         <is>
           <t>Rejected - Skill Gap</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="33.95" customHeight="1" s="17">
-      <c r="A59" s="13" t="inlineStr">
+    <row r="59" ht="33.95" customHeight="1" s="20">
+      <c r="A59" s="11" t="inlineStr">
         <is>
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="B59" s="13" t="inlineStr">
+      <c r="B59" s="11" t="inlineStr">
         <is>
           <t>Persistent Systems (Direct Portal)</t>
         </is>
       </c>
-      <c r="C59" s="13" t="inlineStr">
+      <c r="C59" s="11" t="inlineStr">
         <is>
           <t>Sr Data Engineer (Job Code 177204)</t>
         </is>
       </c>
-      <c r="D59" s="13" t="inlineStr">
+      <c r="D59" s="11" t="inlineStr">
         <is>
           <t>PAN India</t>
         </is>
       </c>
-      <c r="E59" s="13" t="inlineStr">
+      <c r="E59" s="11" t="inlineStr">
         <is>
           <t>Direct Portal</t>
         </is>
       </c>
-      <c r="F59" s="13" t="n">
+      <c r="F59" s="25" t="n">
         <v>0.55</v>
       </c>
-      <c r="G59" s="13" t="inlineStr">
+      <c r="G59" s="11" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="H59" s="13" t="inlineStr">
+      <c r="H59" s="11" t="inlineStr">
         <is>
           <t>Not Applied - Skill Gap</t>
         </is>
       </c>
-      <c r="I59" s="13" t="n"/>
-      <c r="J59" s="13" t="n"/>
-      <c r="K59" s="13" t="inlineStr">
+      <c r="I59" s="11" t="n"/>
+      <c r="J59" s="11" t="n"/>
+      <c r="K59" s="11" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="L59" s="13" t="n"/>
-      <c r="M59" s="13" t="inlineStr">
+      <c r="L59" s="11" t="n"/>
+      <c r="M59" s="11" t="inlineStr">
         <is>
           <t>Not Specified</t>
         </is>
       </c>
-      <c r="N59" s="13" t="inlineStr">
+      <c r="N59" s="11" t="inlineStr">
         <is>
           <t>JD reviewed. Major gaps: PySpark, Apache Spark, Kafka, Dell Boomi. Different from Growel Softech Persistent JD (SQL+Snowflake+DBT). Not applied.</t>
         </is>
       </c>
-      <c r="O59" s="13" t="inlineStr">
+      <c r="O59" s="11" t="inlineStr">
         <is>
           <t>Rejected - Skill Gap</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="33.95" customHeight="1" s="17">
-      <c r="A60" s="14" t="inlineStr">
+    <row r="60" ht="33.95" customHeight="1" s="20">
+      <c r="A60" s="12" t="inlineStr">
         <is>
           <t>2026-08-05</t>
         </is>
       </c>
-      <c r="B60" s="14" t="inlineStr">
+      <c r="B60" s="12" t="inlineStr">
         <is>
           <t>Magellanic Cloud (IBM/SAP Client)</t>
         </is>
       </c>
-      <c r="C60" s="14" t="inlineStr">
+      <c r="C60" s="12" t="inlineStr">
         <is>
           <t>Data Engineer</t>
         </is>
       </c>
-      <c r="D60" s="14" t="inlineStr">
+      <c r="D60" s="12" t="inlineStr">
         <is>
           <t>Hyderabad / Remote</t>
         </is>
       </c>
-      <c r="E60" s="14" t="inlineStr">
+      <c r="E60" s="12" t="inlineStr">
         <is>
           <t>Naukri Outreach</t>
         </is>
       </c>
-      <c r="F60" s="14" t="n">
+      <c r="F60" s="26" t="n">
         <v>0.85</v>
       </c>
-      <c r="G60" s="14" t="inlineStr">
+      <c r="G60" s="12" t="inlineStr">
         <is>
           <t>M_Haresh_Kumar_Data_SQL_DBT_PowerBI_Resume.pdf</t>
         </is>
       </c>
-      <c r="H60" s="21" t="inlineStr">
+      <c r="H60" s="16" t="inlineStr">
         <is>
           <t>IBM AI Talent Matching Consent Confirmed</t>
         </is>
       </c>
-      <c r="I60" s="14" t="inlineStr">
+      <c r="I60" s="12" t="inlineStr">
         <is>
           <t>Vindhya BV</t>
         </is>
       </c>
-      <c r="J60" s="14" t="inlineStr">
+      <c r="J60" s="12" t="inlineStr">
         <is>
           <t>9483490498</t>
         </is>
       </c>
-      <c r="K60" s="14" t="inlineStr">
+      <c r="K60" s="12" t="inlineStr">
         <is>
           <t>Candidate completed IBM Talent Acquisition AI matching consent form on Aug 10. Profile registered in IBM global candidate matching database.</t>
         </is>
       </c>
-      <c r="L60" s="14" t="inlineStr">
+      <c r="L60" s="12" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
       </c>
-      <c r="M60" s="14" t="inlineStr">
+      <c r="M60" s="12" t="inlineStr">
         <is>
           <t>9 LPA Current / 14-15 LPA Expected</t>
         </is>
       </c>
-      <c r="N60" s="14" t="inlineStr">
+      <c r="N60" s="12" t="inlineStr">
         <is>
           <t>Confirmed consent on IBM Talent Acquisition AI profile matching form on Aug 10.</t>
         </is>
       </c>
-      <c r="O60" s="14" t="inlineStr">
+      <c r="O60" s="12" t="inlineStr">
         <is>
           <t>Closed - Skill Gap</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="33.95" customHeight="1" s="17">
-      <c r="A61" s="14" t="inlineStr">
+    <row r="61" ht="33.95" customHeight="1" s="20">
+      <c r="A61" s="12" t="inlineStr">
         <is>
           <t>2026-08-05</t>
         </is>
       </c>
-      <c r="B61" s="14" t="inlineStr">
+      <c r="B61" s="12" t="inlineStr">
         <is>
           <t>Vn Software (Client: Wells Fargo Req 1191)</t>
         </is>
       </c>
-      <c r="C61" s="14" t="inlineStr">
+      <c r="C61" s="12" t="inlineStr">
         <is>
           <t>Data Governance / Data Quality Analyst</t>
         </is>
       </c>
-      <c r="D61" s="14" t="inlineStr">
+      <c r="D61" s="12" t="inlineStr">
         <is>
           <t>Bengaluru (Wells Fargo Enterprise Data Governance Group)</t>
         </is>
       </c>
-      <c r="E61" s="14" t="inlineStr">
+      <c r="E61" s="12" t="inlineStr">
         <is>
           <t>Naukri Outreach</t>
         </is>
       </c>
-      <c r="F61" s="14" t="n">
+      <c r="F61" s="26" t="n">
         <v>0.8</v>
       </c>
-      <c r="G61" s="14" t="inlineStr">
+      <c r="G61" s="12" t="inlineStr">
         <is>
           <t>M_Haresh_Kumar_Data_SQL_DBT_PowerBI_Resume.pdf</t>
         </is>
       </c>
-      <c r="H61" s="20" t="inlineStr">
+      <c r="H61" s="15" t="inlineStr">
         <is>
           <t>Interview - L1 Pending Feedback (VNest Req 1191)</t>
         </is>
       </c>
-      <c r="I61" s="14" t="inlineStr">
+      <c r="I61" s="12" t="inlineStr">
         <is>
           <t>Snehal Girase / Anjali Jadhav (Vn Software)</t>
         </is>
       </c>
-      <c r="J61" s="14" t="inlineStr">
+      <c r="J61" s="12" t="inlineStr">
         <is>
           <t>9225091789 / 9225091793</t>
         </is>
       </c>
-      <c r="K61" s="14" t="inlineStr">
+      <c r="K61" s="12" t="inlineStr">
         <is>
           <t>VNest Activity Log Verified: Applied Aug 5, L1 Interview scheduled Aug 6 @ 11:00 AM. Status: Interview - L1 Pending Feedback for Wells Fargo Data Quality Analyst (9 Openings).</t>
         </is>
       </c>
-      <c r="L61" s="14" t="inlineStr">
+      <c r="L61" s="12" t="inlineStr">
         <is>
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="M61" s="14" t="inlineStr">
+      <c r="M61" s="12" t="inlineStr">
         <is>
           <t>Not Specified</t>
         </is>
       </c>
-      <c r="N61" s="14" t="inlineStr">
+      <c r="N61" s="12" t="inlineStr">
         <is>
           <t>VNest Activity Log audit: Candidate file submitted Aug 5, L1 Interview milestone logged Aug 6 @ 11:00 AM. Awaiting feedback score entry from panel.</t>
         </is>
       </c>
-      <c r="O61" s="14" t="inlineStr">
+      <c r="O61" s="12" t="inlineStr">
         <is>
           <t>Active - L1 Scheduled</t>
         </is>
       </c>
     </row>
-    <row r="62" ht="33.95" customHeight="1" s="17">
-      <c r="A62" s="14" t="inlineStr">
+    <row r="62" ht="33.95" customHeight="1" s="20">
+      <c r="A62" s="12" t="inlineStr">
         <is>
           <t>2026-08-05</t>
         </is>
       </c>
-      <c r="B62" s="14" t="inlineStr">
+      <c r="B62" s="12" t="inlineStr">
         <is>
           <t>MBIT Computraining (Client: TCS)</t>
         </is>
       </c>
-      <c r="C62" s="14" t="inlineStr">
+      <c r="C62" s="12" t="inlineStr">
         <is>
           <t>Data Governance / AI Specialist</t>
         </is>
       </c>
-      <c r="D62" s="14" t="inlineStr">
+      <c r="D62" s="12" t="inlineStr">
         <is>
           <t>Bengaluru / Hyderabad</t>
         </is>
       </c>
-      <c r="E62" s="14" t="inlineStr">
+      <c r="E62" s="12" t="inlineStr">
         <is>
           <t>Naukri Email Outreach</t>
         </is>
       </c>
-      <c r="F62" s="14" t="n">
+      <c r="F62" s="26" t="n">
         <v>0.9</v>
       </c>
-      <c r="G62" s="14" t="inlineStr">
+      <c r="G62" s="12" t="inlineStr">
         <is>
           <t>M_Haresh_Kumar_Data_Governance_SQL_DBT_PowerBI_Resume.pdf</t>
         </is>
       </c>
-      <c r="H62" s="13" t="inlineStr">
+      <c r="H62" s="11" t="inlineStr">
         <is>
           <t>Closed - Degree Criteria</t>
         </is>
       </c>
-      <c r="I62" s="14" t="inlineStr">
+      <c r="I62" s="12" t="inlineStr">
         <is>
           <t>Kajal (MBIT Computraining)</t>
         </is>
       </c>
-      <c r="J62" s="14" t="inlineStr">
+      <c r="J62" s="12" t="inlineStr">
         <is>
           <t>9311946565</t>
         </is>
       </c>
-      <c r="K62" s="14" t="inlineStr">
+      <c r="K62" s="12" t="inlineStr">
         <is>
           <t>Agreed to 11-12 LPA Budget. Updated Data Governance resume sent to Kajal via WhatsApp.</t>
         </is>
       </c>
-      <c r="L62" s="14" t="inlineStr">
+      <c r="L62" s="12" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
       </c>
-      <c r="M62" s="14" t="inlineStr">
+      <c r="M62" s="12" t="inlineStr">
         <is>
           <t>Current 9 LPA / Expected 14-15 LPA</t>
         </is>
       </c>
-      <c r="N62" s="14" t="inlineStr">
+      <c r="N62" s="12" t="inlineStr">
         <is>
           <t>Recruiter (Kajal) informed TCS requires mandatory completed degree. Candidate transparently shared KSOU 2013-2016 UGC issue &amp; NIOS status. Closed due to client policy filter.</t>
         </is>
       </c>
-      <c r="O62" s="14" t="inlineStr">
+      <c r="O62" s="12" t="inlineStr">
         <is>
           <t>Closed - Degree Criteria</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="33.95" customHeight="1" s="17">
-      <c r="A63" s="14" t="inlineStr">
+    <row r="63" ht="33.95" customHeight="1" s="20">
+      <c r="A63" s="12" t="inlineStr">
         <is>
           <t>2026-08-02</t>
         </is>
       </c>
-      <c r="B63" s="14" t="inlineStr">
+      <c r="B63" s="12" t="inlineStr">
         <is>
           <t>Yukthi Systems</t>
         </is>
       </c>
-      <c r="C63" s="14" t="inlineStr">
+      <c r="C63" s="12" t="inlineStr">
         <is>
           <t>Head of Data Operations</t>
         </is>
       </c>
-      <c r="D63" s="14" t="inlineStr">
+      <c r="D63" s="12" t="inlineStr">
         <is>
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="E63" s="14" t="inlineStr">
+      <c r="E63" s="12" t="inlineStr">
         <is>
           <t>Naukri / Direct</t>
         </is>
       </c>
-      <c r="F63" s="14" t="n">
+      <c r="F63" s="26" t="n">
         <v>0.95</v>
       </c>
-      <c r="G63" s="14" t="inlineStr">
-        <is>
-          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
-        </is>
-      </c>
-      <c r="H63" s="14" t="inlineStr">
+      <c r="G63" s="12" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H63" s="12" t="inlineStr">
         <is>
           <t>Applied (3d ago)</t>
         </is>
       </c>
-      <c r="I63" s="14" t="inlineStr">
+      <c r="I63" s="12" t="inlineStr">
         <is>
           <t>Managing Director (Yukthi Systems)</t>
         </is>
       </c>
-      <c r="J63" s="14" t="inlineStr">
+      <c r="J63" s="12" t="inlineStr">
         <is>
           <t>Naukri NVite</t>
         </is>
       </c>
-      <c r="K63" s="14" t="inlineStr">
+      <c r="K63" s="12" t="inlineStr">
         <is>
           <t>Application Submitted (3d ago) → NVite Sent</t>
         </is>
       </c>
-      <c r="L63" s="14" t="inlineStr">
+      <c r="L63" s="12" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
       </c>
-      <c r="M63" s="14" t="inlineStr">
+      <c r="M63" s="12" t="inlineStr">
         <is>
           <t>Not Specified (Target 15-18 LPA)</t>
         </is>
       </c>
-      <c r="N63" s="14" t="inlineStr">
+      <c r="N63" s="12" t="inlineStr">
         <is>
           <t>Head of Data Operations role applied 3 days ago. Recruiter / MD sent NVite on Naukri.</t>
         </is>
       </c>
-      <c r="O63" s="14" t="inlineStr">
+      <c r="O63" s="12" t="inlineStr">
         <is>
           <t>Active - Applied</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="33.95" customHeight="1" s="17">
-      <c r="A64" s="20" t="inlineStr">
+    <row r="64" ht="33.95" customHeight="1" s="20">
+      <c r="A64" s="15" t="inlineStr">
         <is>
           <t>2026-08-01</t>
         </is>
       </c>
-      <c r="B64" s="20" t="inlineStr">
+      <c r="B64" s="15" t="inlineStr">
         <is>
           <t>Flipkart (Flipkart Minutes)</t>
         </is>
       </c>
-      <c r="C64" s="20" t="inlineStr">
+      <c r="C64" s="15" t="inlineStr">
         <is>
           <t>Senior Manager - Data &amp; Analytics</t>
         </is>
       </c>
-      <c r="D64" s="20" t="inlineStr">
+      <c r="D64" s="15" t="inlineStr">
         <is>
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="E64" s="20" t="inlineStr">
+      <c r="E64" s="15" t="inlineStr">
         <is>
           <t>LinkedIn Inbound Network (Basavaraj)</t>
         </is>
       </c>
-      <c r="F64" s="20" t="n">
+      <c r="F64" s="27" t="n">
         <v>0.95</v>
       </c>
-      <c r="G64" s="20" t="inlineStr">
-        <is>
-          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
-        </is>
-      </c>
-      <c r="H64" s="21" t="inlineStr">
+      <c r="G64" s="15" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H64" s="16" t="inlineStr">
         <is>
           <t>Closed - Role Filled (Amazon Hired)</t>
         </is>
       </c>
-      <c r="I64" s="20" t="inlineStr">
+      <c r="I64" s="15" t="inlineStr">
         <is>
           <t>Basavaraj (Data Analyst @ Flipkart Minutes)</t>
         </is>
       </c>
-      <c r="J64" s="20" t="inlineStr">
+      <c r="J64" s="15" t="inlineStr">
         <is>
           <t>7676035429</t>
         </is>
       </c>
-      <c r="K64" s="20" t="inlineStr">
+      <c r="K64" s="15" t="inlineStr">
         <is>
           <t>Inbound reachout on WhatsApp by Basavaraj. Offered to check/refer for Senior Manager Data role at Flipkart Minutes.</t>
         </is>
       </c>
-      <c r="L64" s="20" t="inlineStr">
+      <c r="L64" s="15" t="inlineStr">
         <is>
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="M64" s="20" t="inlineStr">
+      <c r="M64" s="15" t="inlineStr">
         <is>
           <t>Target 18-22 LPA</t>
         </is>
       </c>
-      <c r="N64" s="20" t="inlineStr">
+      <c r="N64" s="15" t="inlineStr">
         <is>
           <t>Basavaraj (Flipkart Minutes) confirmed on WhatsApp on Aug 5 that the Senior Manager position was filled internally/externally by an Amazon candidate. Referral closed.</t>
         </is>
       </c>
-      <c r="O64" s="20" t="inlineStr">
+      <c r="O64" s="15" t="inlineStr">
         <is>
           <t>Closed - Role Filled</t>
         </is>
       </c>
     </row>
-    <row r="65" ht="33.95" customHeight="1" s="17">
-      <c r="A65" s="20" t="inlineStr">
+    <row r="65" ht="33.95" customHeight="1" s="20">
+      <c r="A65" s="15" t="inlineStr">
         <is>
           <t>2026-08-05</t>
         </is>
       </c>
-      <c r="B65" s="20" t="inlineStr">
+      <c r="B65" s="15" t="inlineStr">
         <is>
           <t>Quinnox (Everforth Quinnox)</t>
         </is>
       </c>
-      <c r="C65" s="20" t="inlineStr">
+      <c r="C65" s="15" t="inlineStr">
         <is>
           <t>Senior Manager - Power BI &amp; SQL</t>
         </is>
       </c>
-      <c r="D65" s="20" t="inlineStr">
+      <c r="D65" s="15" t="inlineStr">
         <is>
           <t>Bengaluru (Hybrid)</t>
         </is>
       </c>
-      <c r="E65" s="20" t="inlineStr">
+      <c r="E65" s="15" t="inlineStr">
         <is>
           <t>Naukri Urgent Direct Post</t>
         </is>
       </c>
-      <c r="F65" s="20" t="n">
+      <c r="F65" s="27" t="n">
         <v>0.98</v>
       </c>
-      <c r="G65" s="20" t="inlineStr">
-        <is>
-          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
-        </is>
-      </c>
-      <c r="H65" s="20" t="inlineStr">
+      <c r="G65" s="15" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H65" s="15" t="inlineStr">
         <is>
           <t>Submitted</t>
         </is>
       </c>
-      <c r="I65" s="20" t="inlineStr">
+      <c r="I65" s="15" t="inlineStr">
         <is>
           <t>Quinnox Hiring Team</t>
         </is>
       </c>
-      <c r="J65" s="20" t="inlineStr">
+      <c r="J65" s="15" t="inlineStr">
         <is>
           <t>Naukri Direct</t>
         </is>
       </c>
-      <c r="K65" s="20" t="inlineStr">
+      <c r="K65" s="15" t="inlineStr">
         <is>
           <t>Application logged. Requirements: 12+ Yrs Exp, Immediate Joiner, Power BI DAX, Scorecards, SQL stored procedures, CTEs, Window functions.</t>
         </is>
       </c>
-      <c r="L65" s="20" t="inlineStr">
+      <c r="L65" s="15" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
       </c>
-      <c r="M65" s="20" t="inlineStr">
+      <c r="M65" s="15" t="inlineStr">
         <is>
           <t>Target 16-20 LPA</t>
         </is>
       </c>
-      <c r="N65" s="20" t="inlineStr">
+      <c r="N65" s="15" t="inlineStr">
         <is>
           <t>Naukri direct opening for Senior Manager Power BI &amp; SQL at Quinnox Bangalore. 12+ Yrs Exp, Immediate Joiner requirement. 100% skill match.</t>
         </is>
       </c>
-      <c r="O65" s="20" t="inlineStr">
+      <c r="O65" s="15" t="inlineStr">
         <is>
           <t>Active - Submitted</t>
         </is>
       </c>
     </row>
-    <row r="66" ht="33.95" customHeight="1" s="17">
+    <row r="66" ht="33.95" customHeight="1" s="20">
       <c r="A66" t="inlineStr">
         <is>
           <t>2026-08-07</t>
@@ -4862,7 +4882,7 @@
           <t>Naukri Invite (Vaishnava J)</t>
         </is>
       </c>
-      <c r="F66" t="n">
+      <c r="F66" s="28" t="n">
         <v>0.75</v>
       </c>
       <c r="G66" t="inlineStr">
@@ -4911,82 +4931,82 @@
         </is>
       </c>
     </row>
-    <row r="67" ht="33.95" customHeight="1" s="17">
-      <c r="A67" s="20" t="inlineStr">
+    <row r="67" ht="33.95" customHeight="1" s="20">
+      <c r="A67" s="15" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
       </c>
-      <c r="B67" s="20" t="inlineStr">
+      <c r="B67" s="15" t="inlineStr">
         <is>
           <t>Mars Technominds Inc</t>
         </is>
       </c>
-      <c r="C67" s="20" t="inlineStr">
+      <c r="C67" s="15" t="inlineStr">
         <is>
           <t>Senior / Lead Power BI Developer</t>
         </is>
       </c>
-      <c r="D67" s="20" t="inlineStr">
+      <c r="D67" s="15" t="inlineStr">
         <is>
           <t>Hyderabad (In-Office)</t>
         </is>
       </c>
-      <c r="E67" s="20" t="inlineStr">
+      <c r="E67" s="15" t="inlineStr">
         <is>
           <t>Naukri Invite (Mars Technominds)</t>
         </is>
       </c>
-      <c r="F67" s="20" t="n">
+      <c r="F67" s="27" t="n">
         <v>0.98</v>
       </c>
-      <c r="G67" s="20" t="inlineStr">
-        <is>
-          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
-        </is>
-      </c>
-      <c r="H67" s="20" t="inlineStr">
+      <c r="G67" s="15" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H67" s="15" t="inlineStr">
         <is>
           <t>Application &amp; Profile Viewed by Recruiter</t>
         </is>
       </c>
-      <c r="I67" s="20" t="inlineStr">
+      <c r="I67" s="15" t="inlineStr">
         <is>
           <t>Mars Technominds Hiring Team</t>
         </is>
       </c>
-      <c r="J67" s="20" t="inlineStr">
+      <c r="J67" s="15" t="inlineStr">
         <is>
           <t>Naukri Direct Invite</t>
         </is>
       </c>
-      <c r="K67" s="20" t="inlineStr">
+      <c r="K67" s="15" t="inlineStr">
         <is>
           <t>Mars Technominds recruiter (Harika) viewed profile &amp; application on Naukri on Aug 7.</t>
         </is>
       </c>
-      <c r="L67" s="20" t="inlineStr">
+      <c r="L67" s="15" t="inlineStr">
         <is>
           <t>2026-08-09</t>
         </is>
       </c>
-      <c r="M67" s="20" t="inlineStr">
+      <c r="M67" s="15" t="inlineStr">
         <is>
           <t>Target 14-17 LPA</t>
         </is>
       </c>
-      <c r="N67" s="20" t="inlineStr">
+      <c r="N67" s="15" t="inlineStr">
         <is>
           <t>Mars Technominds HR viewed application on Naukri for Senior/Lead Power BI Developer (7.0 - 17.0 LPA, Hyderabad). Profile active in screening pipeline.</t>
         </is>
       </c>
-      <c r="O67" s="20" t="inlineStr">
+      <c r="O67" s="15" t="inlineStr">
         <is>
           <t>Active - Target Applied</t>
         </is>
       </c>
     </row>
-    <row r="68" ht="33.95" customHeight="1" s="17">
+    <row r="68" ht="33.95" customHeight="1" s="20">
       <c r="A68" t="inlineStr">
         <is>
           <t>2026-08-07</t>
@@ -5012,7 +5032,7 @@
           <t>Naukri Profile View (Ritika - Head HR)</t>
         </is>
       </c>
-      <c r="F68" t="n">
+      <c r="F68" s="28" t="n">
         <v>0.85</v>
       </c>
       <c r="G68" t="inlineStr">
@@ -5061,7 +5081,7 @@
         </is>
       </c>
     </row>
-    <row r="69" ht="33.95" customHeight="1" s="17">
+    <row r="69" ht="33.95" customHeight="1" s="20">
       <c r="A69" t="inlineStr">
         <is>
           <t>2026-08-07</t>
@@ -5087,7 +5107,7 @@
           <t>Naukri Direct Invite (Aruna M / ZettaMine)</t>
         </is>
       </c>
-      <c r="F69" t="n">
+      <c r="F69" s="28" t="n">
         <v>0.7</v>
       </c>
       <c r="G69" t="inlineStr">
@@ -5136,157 +5156,157 @@
         </is>
       </c>
     </row>
-    <row r="70" ht="33.95" customHeight="1" s="17">
-      <c r="A70" s="20" t="inlineStr">
+    <row r="70" ht="33.95" customHeight="1" s="20">
+      <c r="A70" s="15" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
       </c>
-      <c r="B70" s="20" t="inlineStr">
+      <c r="B70" s="15" t="inlineStr">
         <is>
           <t>AECOM</t>
         </is>
       </c>
-      <c r="C70" s="20" t="inlineStr">
+      <c r="C70" s="15" t="inlineStr">
         <is>
           <t>Data Analytics and Reporting Lead</t>
         </is>
       </c>
-      <c r="D70" s="20" t="inlineStr">
+      <c r="D70" s="15" t="inlineStr">
         <is>
           <t>Bengaluru (Hybrid)</t>
         </is>
       </c>
-      <c r="E70" s="20" t="inlineStr">
+      <c r="E70" s="15" t="inlineStr">
         <is>
           <t>LinkedIn Alert (AECOM)</t>
         </is>
       </c>
-      <c r="F70" s="20" t="n">
+      <c r="F70" s="27" t="n">
         <v>0.98</v>
       </c>
-      <c r="G70" s="20" t="inlineStr">
-        <is>
-          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
-        </is>
-      </c>
-      <c r="H70" s="20" t="inlineStr">
+      <c r="G70" s="15" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H70" s="15" t="inlineStr">
         <is>
           <t>Submitted / Target Applied</t>
         </is>
       </c>
-      <c r="I70" s="20" t="inlineStr">
+      <c r="I70" s="15" t="inlineStr">
         <is>
           <t>AECOM Talent Acquisition</t>
         </is>
       </c>
-      <c r="J70" s="20" t="inlineStr">
+      <c r="J70" s="15" t="inlineStr">
         <is>
           <t>LinkedIn Direct</t>
         </is>
       </c>
-      <c r="K70" s="20" t="inlineStr">
+      <c r="K70" s="15" t="inlineStr">
         <is>
           <t>100% Core Lead Skill Match. Requirements: Data Analytics &amp; Reporting Lead, Bengaluru, Power BI, SQL, Executive Reporting.</t>
         </is>
       </c>
-      <c r="L70" s="20" t="inlineStr">
+      <c r="L70" s="15" t="inlineStr">
         <is>
           <t>2026-08-09</t>
         </is>
       </c>
-      <c r="M70" s="20" t="inlineStr">
+      <c r="M70" s="15" t="inlineStr">
         <is>
           <t>Target 16-20 LPA</t>
         </is>
       </c>
-      <c r="N70" s="20" t="inlineStr">
+      <c r="N70" s="15" t="inlineStr">
         <is>
           <t>LinkedIn Job Alert: Data Analytics and Reporting Lead at AECOM Bangalore. 100% skill match (Power BI, SQL, Reporting Leadership).</t>
         </is>
       </c>
-      <c r="O70" s="20" t="inlineStr">
+      <c r="O70" s="15" t="inlineStr">
         <is>
           <t>Active - Target Applied</t>
         </is>
       </c>
     </row>
-    <row r="71" ht="33.95" customHeight="1" s="17">
-      <c r="A71" s="20" t="inlineStr">
+    <row r="71" ht="33.95" customHeight="1" s="20">
+      <c r="A71" s="15" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
       </c>
-      <c r="B71" s="20" t="inlineStr">
+      <c r="B71" s="15" t="inlineStr">
         <is>
           <t>NetApp</t>
         </is>
       </c>
-      <c r="C71" s="20" t="inlineStr">
+      <c r="C71" s="15" t="inlineStr">
         <is>
           <t>Business Analyst (Data &amp; Finance Analytics)</t>
         </is>
       </c>
-      <c r="D71" s="20" t="inlineStr">
+      <c r="D71" s="15" t="inlineStr">
         <is>
           <t>Bengaluru (Hybrid)</t>
         </is>
       </c>
-      <c r="E71" s="20" t="inlineStr">
+      <c r="E71" s="15" t="inlineStr">
         <is>
           <t>LinkedIn Direct (NetApp Portal)</t>
         </is>
       </c>
-      <c r="F71" s="20" t="n">
+      <c r="F71" s="27" t="n">
         <v>0.95</v>
       </c>
-      <c r="G71" s="20" t="inlineStr">
-        <is>
-          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
-        </is>
-      </c>
-      <c r="H71" s="20" t="inlineStr">
-        <is>
-          <t>Reviewed - Target Selected for Applied Queue</t>
-        </is>
-      </c>
-      <c r="I71" s="20" t="inlineStr">
+      <c r="G71" s="15" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H71" s="15" t="inlineStr">
+        <is>
+          <t>Reviewed - Skipped (Domain Skill Gap: Finance Analytics)</t>
+        </is>
+      </c>
+      <c r="I71" s="15" t="inlineStr">
         <is>
           <t>NetApp Talent Acquisition</t>
         </is>
       </c>
-      <c r="J71" s="20" t="inlineStr">
+      <c r="J71" s="15" t="inlineStr">
         <is>
           <t>NetApp Careers Portal</t>
         </is>
       </c>
-      <c r="K71" s="20" t="inlineStr">
+      <c r="K71" s="15" t="inlineStr">
         <is>
           <t>95% Skill Match. Requirements: Power BI, Advanced Excel, SQL, Data Models, Data Quality, Automated Scorecards, EDW Reporting.</t>
         </is>
       </c>
-      <c r="L71" s="20" t="inlineStr">
+      <c r="L71" s="15" t="inlineStr">
         <is>
           <t>2026-08-09</t>
         </is>
       </c>
-      <c r="M71" s="20" t="inlineStr">
+      <c r="M71" s="15" t="inlineStr">
         <is>
           <t>Target 16-22 LPA</t>
         </is>
       </c>
-      <c r="N71" s="20" t="inlineStr">
-        <is>
-          <t>Target role selected from NetApp Workday careers portal for Business Analyst (Data &amp; Finance Analytics). Pending direct web form submission.</t>
-        </is>
-      </c>
-      <c r="O71" s="20" t="inlineStr">
+      <c r="N71" s="15" t="inlineStr">
+        <is>
+          <t>Reviewed - Skipped per candidate instruction (Domain skill gap: required specialized Finance Analytics background).</t>
+        </is>
+      </c>
+      <c r="O71" s="15" t="inlineStr">
         <is>
           <t>Active - Target Applied</t>
         </is>
       </c>
     </row>
-    <row r="72" ht="33.95" customHeight="1" s="17">
+    <row r="72" ht="33.95" customHeight="1" s="20">
       <c r="A72" t="inlineStr">
         <is>
           <t>2026-08-07</t>
@@ -5312,7 +5332,7 @@
           <t>LinkedIn Easy Apply (Chetan Gurudev)</t>
         </is>
       </c>
-      <c r="F72" t="n">
+      <c r="F72" s="28" t="n">
         <v>0.65</v>
       </c>
       <c r="G72" t="inlineStr">
@@ -5361,157 +5381,157 @@
         </is>
       </c>
     </row>
-    <row r="73" ht="33.95" customHeight="1" s="17">
-      <c r="A73" s="20" t="inlineStr">
+    <row r="73" ht="33.95" customHeight="1" s="20">
+      <c r="A73" s="15" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
       </c>
-      <c r="B73" s="20" t="inlineStr">
+      <c r="B73" s="15" t="inlineStr">
         <is>
           <t>BCforward</t>
         </is>
       </c>
-      <c r="C73" s="20" t="inlineStr">
+      <c r="C73" s="15" t="inlineStr">
         <is>
           <t>Snowflake Data Warehouse &amp; Power BI Engineer</t>
         </is>
       </c>
-      <c r="D73" s="20" t="inlineStr">
+      <c r="D73" s="15" t="inlineStr">
         <is>
           <t>Bengaluru (Hybrid)</t>
         </is>
       </c>
-      <c r="E73" s="20" t="inlineStr">
+      <c r="E73" s="15" t="inlineStr">
         <is>
           <t>LinkedIn Direct Email (Srivastav Ghatti)</t>
         </is>
       </c>
-      <c r="F73" s="20" t="n">
+      <c r="F73" s="27" t="n">
         <v>0.98</v>
       </c>
-      <c r="G73" s="20" t="inlineStr">
-        <is>
-          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
-        </is>
-      </c>
-      <c r="H73" s="20" t="inlineStr">
+      <c r="G73" s="15" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H73" s="15" t="inlineStr">
         <is>
           <t>Direct Email Sent to Recruiter</t>
         </is>
       </c>
-      <c r="I73" s="20" t="inlineStr">
+      <c r="I73" s="15" t="inlineStr">
         <is>
           <t>Srivastav Ghatti (Sr. TA @ BCforward)</t>
         </is>
       </c>
-      <c r="J73" s="20" t="inlineStr">
+      <c r="J73" s="15" t="inlineStr">
         <is>
           <t>srivastav.ghatti@bcforward.com</t>
         </is>
       </c>
-      <c r="K73" s="20" t="inlineStr">
+      <c r="K73" s="15" t="inlineStr">
         <is>
           <t>Direct email application sent to srivastav.ghatti@bcforward.com on Aug 7. 100% Core Skill Match (Snowflake, Power BI, Data Migration, Immediate Joiner).</t>
         </is>
       </c>
-      <c r="L73" s="20" t="inlineStr">
+      <c r="L73" s="15" t="inlineStr">
         <is>
           <t>2026-08-09</t>
         </is>
       </c>
-      <c r="M73" s="20" t="inlineStr">
+      <c r="M73" s="15" t="inlineStr">
         <is>
           <t>Target 16-20 LPA</t>
         </is>
       </c>
-      <c r="N73" s="20" t="inlineStr">
+      <c r="N73" s="15" t="inlineStr">
         <is>
           <t>Sent email with PDF resume to Srivastav Ghatti for Snowflake &amp; Power BI Engineer role (Bangalore/Pune/Hyd, 16-20 LPA).</t>
         </is>
       </c>
-      <c r="O73" s="20" t="inlineStr">
+      <c r="O73" s="15" t="inlineStr">
         <is>
           <t>Active - Email Submitted</t>
         </is>
       </c>
     </row>
-    <row r="74" ht="33.95" customHeight="1" s="17">
-      <c r="A74" s="20" t="inlineStr">
+    <row r="74" ht="33.95" customHeight="1" s="20">
+      <c r="A74" s="15" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
       </c>
-      <c r="B74" s="20" t="inlineStr">
+      <c r="B74" s="15" t="inlineStr">
         <is>
           <t>GyanSys Inc.</t>
         </is>
       </c>
-      <c r="C74" s="20" t="inlineStr">
+      <c r="C74" s="15" t="inlineStr">
         <is>
           <t>Power BI Data Engineer (Fabric &amp; DAX)</t>
         </is>
       </c>
-      <c r="D74" s="20" t="inlineStr">
+      <c r="D74" s="15" t="inlineStr">
         <is>
           <t>Bengaluru (On-site)</t>
         </is>
       </c>
-      <c r="E74" s="20" t="inlineStr">
+      <c r="E74" s="15" t="inlineStr">
         <is>
           <t>LinkedIn Direct Email (Komal K.)</t>
         </is>
       </c>
-      <c r="F74" s="20" t="n">
+      <c r="F74" s="27" t="n">
         <v>0.98</v>
       </c>
-      <c r="G74" s="20" t="inlineStr">
-        <is>
-          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
-        </is>
-      </c>
-      <c r="H74" s="20" t="inlineStr">
+      <c r="G74" s="15" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H74" s="15" t="inlineStr">
         <is>
           <t>Reviewed - Poor Work Culture &amp; Heavy Overtime</t>
         </is>
       </c>
-      <c r="I74" s="20" t="inlineStr">
+      <c r="I74" s="15" t="inlineStr">
         <is>
           <t>Komal Kaithwas (Senior Recruiter)</t>
         </is>
       </c>
-      <c r="J74" s="20" t="inlineStr">
+      <c r="J74" s="15" t="inlineStr">
         <is>
           <t>komal.kaithwas@gyansys.com</t>
         </is>
       </c>
-      <c r="K74" s="20" t="inlineStr">
+      <c r="K74" s="15" t="inlineStr">
         <is>
           <t>100% Core Skill Match. Requirements: Advanced SQL, Dimensional Data Modeling (Star Schema), Power BI DAX, Microsoft Fabric, Python, Data Quality Testing, Immediate Joiner.</t>
         </is>
       </c>
-      <c r="L74" s="20" t="inlineStr">
+      <c r="L74" s="15" t="inlineStr">
         <is>
           <t>2026-08-09</t>
         </is>
       </c>
-      <c r="M74" s="20" t="inlineStr">
+      <c r="M74" s="15" t="inlineStr">
         <is>
           <t>Target 14-18 LPA</t>
         </is>
       </c>
-      <c r="N74" s="20" t="inlineStr">
+      <c r="N74" s="15" t="inlineStr">
         <is>
           <t>Evaluated GyanSys Inc. Low employee ratings (2.7 - 3.1/5) on Glassdoor/AmbitionBox for rigid monitoring, high overtime, and poor work-life balance. Deprioritized.</t>
         </is>
       </c>
-      <c r="O74" s="20" t="inlineStr">
+      <c r="O74" s="15" t="inlineStr">
         <is>
           <t>Reviewed - Deprioritized</t>
         </is>
       </c>
     </row>
-    <row r="75" ht="33.95" customHeight="1" s="17">
+    <row r="75" ht="33.95" customHeight="1" s="20">
       <c r="A75" t="inlineStr">
         <is>
           <t>2026-08-07</t>
@@ -5537,7 +5557,7 @@
           <t>Naukri Invite (TechBlocks)</t>
         </is>
       </c>
-      <c r="F75" t="n">
+      <c r="F75" s="28" t="n">
         <v>0.3</v>
       </c>
       <c r="G75" t="inlineStr">
@@ -5586,7 +5606,7 @@
         </is>
       </c>
     </row>
-    <row r="76" ht="33.95" customHeight="1" s="17">
+    <row r="76" ht="33.95" customHeight="1" s="20">
       <c r="A76" t="inlineStr">
         <is>
           <t>2026-08-07</t>
@@ -5612,7 +5632,7 @@
           <t>LinkedIn Direct (Juniper Square Portal)</t>
         </is>
       </c>
-      <c r="F76" t="n">
+      <c r="F76" s="28" t="n">
         <v>0.4</v>
       </c>
       <c r="G76" t="inlineStr">
@@ -5661,82 +5681,82 @@
         </is>
       </c>
     </row>
-    <row r="77" ht="33.95" customHeight="1" s="17">
-      <c r="A77" s="20" t="inlineStr">
+    <row r="77" ht="33.95" customHeight="1" s="20">
+      <c r="A77" s="15" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
       </c>
-      <c r="B77" s="20" t="inlineStr">
+      <c r="B77" s="15" t="inlineStr">
         <is>
           <t>Blue Cloud Softech Solutions Limited</t>
         </is>
       </c>
-      <c r="C77" s="20" t="inlineStr">
+      <c r="C77" s="15" t="inlineStr">
         <is>
           <t>Power BI &amp; Cloud Data Engineer</t>
         </is>
       </c>
-      <c r="D77" s="20" t="inlineStr">
+      <c r="D77" s="15" t="inlineStr">
         <is>
           <t>Bengaluru (Remote / Hybrid)</t>
         </is>
       </c>
-      <c r="E77" s="20" t="inlineStr">
+      <c r="E77" s="15" t="inlineStr">
         <is>
           <t>LinkedIn Easy Apply (Prasanna Kumar)</t>
         </is>
       </c>
-      <c r="F77" s="20" t="n">
+      <c r="F77" s="27" t="n">
         <v>0.98</v>
       </c>
-      <c r="G77" s="20" t="inlineStr">
-        <is>
-          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
-        </is>
-      </c>
-      <c r="H77" s="20" t="inlineStr">
+      <c r="G77" s="15" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H77" s="15" t="inlineStr">
         <is>
           <t>Skipped / Deprioritized (Heavy Databricks Spark Code Developer)</t>
         </is>
       </c>
-      <c r="I77" s="20" t="inlineStr">
+      <c r="I77" s="15" t="inlineStr">
         <is>
           <t>Prasanna Kumar (Lead Recruiter)</t>
         </is>
       </c>
-      <c r="J77" s="20" t="inlineStr">
+      <c r="J77" s="15" t="inlineStr">
         <is>
           <t>LinkedIn Direct</t>
         </is>
       </c>
-      <c r="K77" s="20" t="inlineStr">
+      <c r="K77" s="15" t="inlineStr">
         <is>
           <t>100% Core Skill Match. Requirements: 60-70% Power BI (DAX, VertiPaq, Star Schema, PL-300), 30-40% Databricks/Delta Lake/Medallion Architecture, SQL Data Quality.</t>
         </is>
       </c>
-      <c r="L77" s="20" t="inlineStr">
+      <c r="L77" s="15" t="inlineStr">
         <is>
           <t>2026-08-09</t>
         </is>
       </c>
-      <c r="M77" s="20" t="inlineStr">
+      <c r="M77" s="15" t="inlineStr">
         <is>
           <t>Target 16-22 LPA</t>
         </is>
       </c>
-      <c r="N77" s="20" t="inlineStr">
+      <c r="N77" s="15" t="inlineStr">
         <is>
           <t>Evaluated Blue Cloud Softech. Secondary 30-40% requirement asks for heavy hands-on Databricks Spark SQL / Scala / Python developer. Skipped per user preference.</t>
         </is>
       </c>
-      <c r="O77" s="20" t="inlineStr">
+      <c r="O77" s="15" t="inlineStr">
         <is>
           <t>Reviewed - Deprioritized</t>
         </is>
       </c>
     </row>
-    <row r="78" ht="33.95" customHeight="1" s="17">
+    <row r="78" ht="33.95" customHeight="1" s="20">
       <c r="A78" t="inlineStr">
         <is>
           <t>2026-08-07</t>
@@ -5762,7 +5782,7 @@
           <t>LinkedIn Direct (Tesco Portal)</t>
         </is>
       </c>
-      <c r="F78" t="n">
+      <c r="F78" s="28" t="n">
         <v>0.45</v>
       </c>
       <c r="G78" t="inlineStr">
@@ -5811,82 +5831,82 @@
         </is>
       </c>
     </row>
-    <row r="79" ht="33.95" customHeight="1" s="17">
-      <c r="A79" s="20" t="inlineStr">
+    <row r="79" ht="33.95" customHeight="1" s="20">
+      <c r="A79" s="15" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
       </c>
-      <c r="B79" s="20" t="inlineStr">
+      <c r="B79" s="15" t="inlineStr">
         <is>
           <t>Owl Ventures (Greenlight Data Platform)</t>
         </is>
       </c>
-      <c r="C79" s="20" t="inlineStr">
+      <c r="C79" s="15" t="inlineStr">
         <is>
           <t>Data Engineer (Snowflake &amp; Data Quality)</t>
         </is>
       </c>
-      <c r="D79" s="20" t="inlineStr">
+      <c r="D79" s="15" t="inlineStr">
         <is>
           <t>Bengaluru (Hybrid)</t>
         </is>
       </c>
-      <c r="E79" s="20" t="inlineStr">
+      <c r="E79" s="15" t="inlineStr">
         <is>
           <t>LinkedIn Direct (Greenlight Portal)</t>
         </is>
       </c>
-      <c r="F79" s="20" t="n">
+      <c r="F79" s="27" t="n">
         <v>0.92</v>
       </c>
-      <c r="G79" s="20" t="inlineStr">
+      <c r="G79" s="15" t="inlineStr">
         <is>
           <t>M_Haresh_Kumar_Data_SQL_DBT_PowerBI_Resume.pdf</t>
         </is>
       </c>
-      <c r="H79" s="20" t="inlineStr">
+      <c r="H79" s="15" t="inlineStr">
         <is>
           <t>Application Submitted &amp; Confirmed</t>
         </is>
       </c>
-      <c r="I79" s="20" t="inlineStr">
+      <c r="I79" s="15" t="inlineStr">
         <is>
           <t>Owl Ventures / Greenlight TA</t>
         </is>
       </c>
-      <c r="J79" s="20" t="inlineStr">
+      <c r="J79" s="15" t="inlineStr">
         <is>
           <t>Greenlight Careers Portal</t>
         </is>
       </c>
-      <c r="K79" s="20" t="inlineStr">
+      <c r="K79" s="15" t="inlineStr">
         <is>
           <t>Application submitted on Greenlight Lever ATS. Official confirmation email received from no-reply@hire.lever.co on Aug 7 at 3:07 PM.</t>
         </is>
       </c>
-      <c r="L79" s="20" t="inlineStr">
+      <c r="L79" s="15" t="inlineStr">
         <is>
           <t>2026-08-09</t>
         </is>
       </c>
-      <c r="M79" s="20" t="inlineStr">
+      <c r="M79" s="15" t="inlineStr">
         <is>
           <t>Target 16-22 LPA</t>
         </is>
       </c>
-      <c r="N79" s="20" t="inlineStr">
+      <c r="N79" s="15" t="inlineStr">
         <is>
           <t>Received official ATS confirmation email from Greenlight Recruiting Team (no-reply@hire.lever.co) for Data Engineer role.</t>
         </is>
       </c>
-      <c r="O79" s="20" t="inlineStr">
+      <c r="O79" s="15" t="inlineStr">
         <is>
           <t>Active - Target Applied</t>
         </is>
       </c>
     </row>
-    <row r="80" ht="33.95" customHeight="1" s="17">
+    <row r="80" ht="33.95" customHeight="1" s="20">
       <c r="A80" t="inlineStr">
         <is>
           <t>2026-08-07</t>
@@ -5912,7 +5932,7 @@
           <t>LinkedIn Direct (Shippeo Portal)</t>
         </is>
       </c>
-      <c r="F80" t="n">
+      <c r="F80" s="28" t="n">
         <v>0.35</v>
       </c>
       <c r="G80" t="inlineStr">
@@ -5961,308 +5981,308 @@
         </is>
       </c>
     </row>
-    <row r="81" ht="33.95" customHeight="1" s="17">
-      <c r="A81" s="20" t="inlineStr">
+    <row r="81" ht="33.95" customHeight="1" s="20">
+      <c r="A81" s="15" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
       </c>
-      <c r="B81" s="20" t="inlineStr">
+      <c r="B81" s="15" t="inlineStr">
         <is>
           <t>Zoho Corporation</t>
         </is>
       </c>
-      <c r="C81" s="20" t="inlineStr">
+      <c r="C81" s="15" t="inlineStr">
         <is>
           <t>Data Operations &amp; Analytics Specialist</t>
         </is>
       </c>
-      <c r="D81" s="20" t="inlineStr">
+      <c r="D81" s="15" t="inlineStr">
         <is>
           <t>Chennai / Bengaluru (Relocation Open)</t>
         </is>
       </c>
-      <c r="E81" s="20" t="inlineStr">
+      <c r="E81" s="15" t="inlineStr">
         <is>
           <t>Zoho Official Careers Portal</t>
         </is>
       </c>
-      <c r="F81" s="20" t="n">
+      <c r="F81" s="27" t="n">
         <v>0.95</v>
       </c>
-      <c r="G81" s="20" t="inlineStr">
-        <is>
-          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
-        </is>
-      </c>
-      <c r="H81" s="20" t="inlineStr">
+      <c r="G81" s="15" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H81" s="15" t="inlineStr">
         <is>
           <t>General Talent Pool Registered (No Active Requisition Match Currently)</t>
         </is>
       </c>
-      <c r="I81" s="20" t="inlineStr">
+      <c r="I81" s="15" t="inlineStr">
         <is>
           <t>Zoho Talent Acquisition</t>
         </is>
       </c>
-      <c r="J81" s="20" t="inlineStr">
+      <c r="J81" s="15" t="inlineStr">
         <is>
           <t>Zoho Careers Portal</t>
         </is>
       </c>
-      <c r="K81" s="20" t="inlineStr">
+      <c r="K81" s="15" t="inlineStr">
         <is>
           <t>Zoho Skills Matrix Submitted: Advanced Excel &amp; Data Validation (14 yrs), SQL / Advanced SQL (3 yrs), Power BI (2 yrs), Snowflake Data Cloud (1 yr), Python &amp; Automation Scripting (1 yr).</t>
         </is>
       </c>
-      <c r="L81" s="20" t="inlineStr">
+      <c r="L81" s="15" t="inlineStr">
         <is>
           <t>2026-08-09</t>
         </is>
       </c>
-      <c r="M81" s="20" t="inlineStr">
+      <c r="M81" s="15" t="inlineStr">
         <is>
           <t>Target 12-16 LPA</t>
         </is>
       </c>
-      <c r="N81" s="20" t="inlineStr">
+      <c r="N81" s="15" t="inlineStr">
         <is>
           <t>Submitted candidate profile on Zoho Careers Portal. System messaged no active matching requisitions currently open; profile registered in Zoho Talent Database.</t>
         </is>
       </c>
-      <c r="O81" s="20" t="inlineStr">
+      <c r="O81" s="15" t="inlineStr">
         <is>
           <t>Active - Talent Pool</t>
         </is>
       </c>
     </row>
-    <row r="82" ht="33.95" customHeight="1" s="17">
-      <c r="A82" s="20" t="inlineStr">
+    <row r="82" ht="33.95" customHeight="1" s="20">
+      <c r="A82" s="15" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
       </c>
-      <c r="B82" s="20" t="inlineStr">
+      <c r="B82" s="15" t="inlineStr">
         <is>
           <t>Euronext</t>
         </is>
       </c>
-      <c r="C82" s="20" t="inlineStr">
+      <c r="C82" s="15" t="inlineStr">
         <is>
           <t>Data &amp; Ops Manager, Rankings</t>
         </is>
       </c>
-      <c r="D82" s="20" t="inlineStr">
+      <c r="D82" s="15" t="inlineStr">
         <is>
           <t>Bengaluru (On-site / UK Shift)</t>
         </is>
       </c>
-      <c r="E82" s="20" t="inlineStr">
+      <c r="E82" s="15" t="inlineStr">
         <is>
           <t>LinkedIn Direct (Euronext Portal)</t>
         </is>
       </c>
-      <c r="F82" s="20" t="n">
+      <c r="F82" s="27" t="n">
         <v>0.99</v>
       </c>
-      <c r="G82" s="20" t="inlineStr">
-        <is>
-          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
-        </is>
-      </c>
-      <c r="H82" s="20" t="inlineStr">
+      <c r="G82" s="15" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H82" s="15" t="inlineStr">
         <is>
           <t>Application Submitted &amp; Confirmed</t>
         </is>
       </c>
-      <c r="I82" s="20" t="inlineStr">
+      <c r="I82" s="15" t="inlineStr">
         <is>
           <t>Euronext Talent Acquisition</t>
         </is>
       </c>
-      <c r="J82" s="20" t="inlineStr">
+      <c r="J82" s="15" t="inlineStr">
         <is>
           <t>Euronext Careers Portal</t>
         </is>
       </c>
-      <c r="K82" s="20" t="inlineStr">
+      <c r="K82" s="15" t="inlineStr">
         <is>
           <t>Official Workday Digest email received from hrhub@myworkday.com (Req R27274 Data &amp; Ops Manager Rankings). Status: Under HR Review.</t>
         </is>
       </c>
-      <c r="L82" s="20" t="inlineStr">
+      <c r="L82" s="15" t="inlineStr">
         <is>
           <t>2026-08-09</t>
         </is>
       </c>
-      <c r="M82" s="20" t="inlineStr">
+      <c r="M82" s="15" t="inlineStr">
         <is>
           <t>Target 18-25 LPA</t>
         </is>
       </c>
-      <c r="N82" s="20" t="inlineStr">
+      <c r="N82" s="15" t="inlineStr">
         <is>
           <t>Euronext Workday Daily Digest email received. Candidate application file R27274 in active HR Business Process review.</t>
         </is>
       </c>
-      <c r="O82" s="20" t="inlineStr">
+      <c r="O82" s="15" t="inlineStr">
         <is>
           <t>Active - Target Applied</t>
         </is>
       </c>
     </row>
-    <row r="83" ht="33.95" customHeight="1" s="17">
-      <c r="A83" s="20" t="inlineStr">
+    <row r="83" ht="33.95" customHeight="1" s="20">
+      <c r="A83" s="15" t="inlineStr">
         <is>
           <t>2026-08-08</t>
         </is>
       </c>
-      <c r="B83" s="20" t="inlineStr">
+      <c r="B83" s="15" t="inlineStr">
         <is>
           <t>Aon</t>
         </is>
       </c>
-      <c r="C83" s="20" t="inlineStr">
+      <c r="C83" s="15" t="inlineStr">
         <is>
           <t>Senior Power BI Architect</t>
         </is>
       </c>
-      <c r="D83" s="20" t="inlineStr">
+      <c r="D83" s="15" t="inlineStr">
         <is>
           <t>Bengaluru (Hybrid)</t>
         </is>
       </c>
-      <c r="E83" s="20" t="inlineStr">
+      <c r="E83" s="15" t="inlineStr">
         <is>
           <t>Naukri Weekend Alert (Aon)</t>
         </is>
       </c>
-      <c r="F83" s="20" t="n">
+      <c r="F83" s="27" t="n">
         <v>0.98</v>
       </c>
-      <c r="G83" s="20" t="inlineStr">
-        <is>
-          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
-        </is>
-      </c>
-      <c r="H83" s="20" t="inlineStr">
+      <c r="G83" s="15" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H83" s="15" t="inlineStr">
         <is>
           <t>Reviewed - Strict Degree Criteria (Full-time Graduate / Post-Graduate Required)</t>
         </is>
       </c>
-      <c r="I83" s="20" t="inlineStr">
+      <c r="I83" s="15" t="inlineStr">
         <is>
           <t>Aon Talent Acquisition</t>
         </is>
       </c>
-      <c r="J83" s="20" t="inlineStr">
+      <c r="J83" s="15" t="inlineStr">
         <is>
           <t>Naukri Direct</t>
         </is>
       </c>
-      <c r="K83" s="20" t="inlineStr">
+      <c r="K83" s="15" t="inlineStr">
         <is>
           <t>100% Core Skill Match. Requirements: Power BI Architecture, DAX, Star Schema Modeling, Performance Tuning, Senior BI Lead.</t>
         </is>
       </c>
-      <c r="L83" s="20" t="inlineStr">
+      <c r="L83" s="15" t="inlineStr">
         <is>
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="M83" s="20" t="inlineStr">
+      <c r="M83" s="15" t="inlineStr">
         <is>
           <t>Target 18-25 LPA</t>
         </is>
       </c>
-      <c r="N83" s="20" t="inlineStr">
+      <c r="N83" s="15" t="inlineStr">
         <is>
           <t>Evaluated Aon Senior Power BI Architect role. Strict requirement asks for mandatory full-time Graduate/Post-Graduate degree. Deprioritized.</t>
         </is>
       </c>
-      <c r="O83" s="20" t="inlineStr">
+      <c r="O83" s="15" t="inlineStr">
         <is>
           <t>Reviewed - Deprioritized</t>
         </is>
       </c>
     </row>
-    <row r="84" ht="33.95" customHeight="1" s="17">
-      <c r="A84" s="20" t="inlineStr">
+    <row r="84" ht="33.95" customHeight="1" s="20">
+      <c r="A84" s="15" t="inlineStr">
         <is>
           <t>2026-08-08</t>
         </is>
       </c>
-      <c r="B84" s="20" t="inlineStr">
+      <c r="B84" s="15" t="inlineStr">
         <is>
           <t>Instatalent Recruit LLP (Client: Foreign MNC)</t>
         </is>
       </c>
-      <c r="C84" s="20" t="inlineStr">
+      <c r="C84" s="15" t="inlineStr">
         <is>
           <t>Data Engineer (Snowflake, Python, dbt)</t>
         </is>
       </c>
-      <c r="D84" s="20" t="inlineStr">
+      <c r="D84" s="15" t="inlineStr">
         <is>
           <t>Bengaluru, Pune, Delhi / NCR</t>
         </is>
       </c>
-      <c r="E84" s="20" t="inlineStr">
+      <c r="E84" s="15" t="inlineStr">
         <is>
           <t>Naukri Recruiter Direct NVite</t>
         </is>
       </c>
-      <c r="F84" s="20" t="n">
+      <c r="F84" s="27" t="n">
         <v>0.95</v>
       </c>
-      <c r="G84" s="20" t="inlineStr">
-        <is>
-          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
-        </is>
-      </c>
-      <c r="H84" s="20" t="inlineStr">
+      <c r="G84" s="15" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H84" s="15" t="inlineStr">
         <is>
           <t>Application Submitted &amp; Confirmed (₹16-22.5 LPA)</t>
         </is>
       </c>
-      <c r="I84" s="20" t="inlineStr">
+      <c r="I84" s="15" t="inlineStr">
         <is>
           <t>Pankaj Saroj (Director @ Instatalent Recruit LLP)</t>
         </is>
       </c>
-      <c r="J84" s="20" t="inlineStr">
+      <c r="J84" s="15" t="inlineStr">
         <is>
           <t>Naukri Direct NVite</t>
         </is>
       </c>
-      <c r="K84" s="20" t="inlineStr">
+      <c r="K84" s="15" t="inlineStr">
         <is>
           <t>100% Core Skill Match. Requirements: Snowflake, Python, dbt (Data Build Tool), Foreign MNC Client, Bangalore/Pune/Delhi, 16.0 - 22.5 LPA.</t>
         </is>
       </c>
-      <c r="L84" s="20" t="inlineStr">
+      <c r="L84" s="15" t="inlineStr">
         <is>
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="M84" s="20" t="inlineStr">
+      <c r="M84" s="15" t="inlineStr">
         <is>
           <t>16.0 - 22.5 LPA</t>
         </is>
       </c>
-      <c r="N84" s="20" t="inlineStr">
+      <c r="N84" s="15" t="inlineStr">
         <is>
           <t>NVite accepted &amp; applied on Naukri for Foreign MNC Data Engineer (₹16.0 - 22.5 LPA). Recruiter: Pankaj Saroj.</t>
         </is>
       </c>
-      <c r="O84" s="20" t="inlineStr">
+      <c r="O84" s="15" t="inlineStr">
         <is>
           <t>Active - Target Applied</t>
         </is>
       </c>
     </row>
-    <row r="85" ht="33.95" customHeight="1" s="17"/>
-    <row r="86" ht="33.95" customHeight="1" s="17">
+    <row r="85" ht="33.95" customHeight="1" s="20"/>
+    <row r="86" ht="33.95" customHeight="1" s="20">
       <c r="A86" t="inlineStr">
         <is>
           <t>2026-08-08</t>
@@ -6299,7 +6319,7 @@
         </is>
       </c>
     </row>
-    <row r="87" ht="33.95" customHeight="1" s="17">
+    <row r="87" ht="33.95" customHeight="1" s="20">
       <c r="A87" t="inlineStr">
         <is>
           <t>2026-08-08</t>
@@ -6336,7 +6356,7 @@
         </is>
       </c>
     </row>
-    <row r="88" ht="33.95" customHeight="1" s="17">
+    <row r="88" ht="33.95" customHeight="1" s="20">
       <c r="A88" t="inlineStr">
         <is>
           <t>2026-08-08</t>
@@ -6362,7 +6382,7 @@
           <t>Naukri Direct (Sahithya Nadella)</t>
         </is>
       </c>
-      <c r="F88" t="n">
+      <c r="F88" s="28" t="n">
         <v>0.98</v>
       </c>
       <c r="G88" t="inlineStr">
@@ -6370,7 +6390,7 @@
           <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
         </is>
       </c>
-      <c r="H88" s="20" t="inlineStr">
+      <c r="H88" s="15" t="inlineStr">
         <is>
           <t>Direct Email Sent to Recruiter (10-20 LPA)</t>
         </is>
@@ -6401,7 +6421,7 @@
         </is>
       </c>
     </row>
-    <row r="89" ht="33.95" customHeight="1" s="17">
+    <row r="89" ht="33.95" customHeight="1" s="20">
       <c r="A89" t="inlineStr">
         <is>
           <t>2026-08-08</t>
@@ -6438,7 +6458,7 @@
         </is>
       </c>
     </row>
-    <row r="90" ht="33.95" customHeight="1" s="17">
+    <row r="90" ht="33.95" customHeight="1" s="20">
       <c r="A90" t="inlineStr">
         <is>
           <t>2026-08-08</t>
@@ -6475,491 +6495,639 @@
         </is>
       </c>
     </row>
-    <row r="91" ht="33.95" customHeight="1" s="17">
-      <c r="A91" s="20" t="inlineStr">
+    <row r="91" ht="33.95" customHeight="1" s="20">
+      <c r="A91" s="15" t="inlineStr">
         <is>
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="B91" s="20" t="inlineStr">
+      <c r="B91" s="15" t="inlineStr">
         <is>
           <t>Recex (Chetna S - Director)</t>
         </is>
       </c>
-      <c r="C91" s="20" t="inlineStr">
+      <c r="C91" s="15" t="inlineStr">
         <is>
           <t>Senior Data / Analytics Opportunity</t>
         </is>
       </c>
-      <c r="D91" s="20" t="inlineStr">
+      <c r="D91" s="15" t="inlineStr">
         <is>
           <t>Kolkata / Remote</t>
         </is>
       </c>
-      <c r="E91" s="20" t="inlineStr">
+      <c r="E91" s="15" t="inlineStr">
         <is>
           <t>Naukri Recruiter Direct NVite</t>
         </is>
       </c>
-      <c r="F91" s="20" t="n">
+      <c r="F91" s="27" t="n">
         <v>0.95</v>
       </c>
-      <c r="G91" s="20" t="inlineStr">
-        <is>
-          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
-        </is>
-      </c>
-      <c r="H91" s="20" t="inlineStr">
+      <c r="G91" s="15" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H91" s="15" t="inlineStr">
         <is>
           <t>Reviewed - Skipped (Strict BE/BTech CS Degree Filter &amp; Heavy Databricks/Scala/DevOps)</t>
         </is>
       </c>
-      <c r="I91" s="20" t="inlineStr">
+      <c r="I91" s="15" t="inlineStr">
         <is>
           <t>Chetna S (Director @ Recex)</t>
         </is>
       </c>
-      <c r="J91" s="20" t="inlineStr">
+      <c r="J91" s="15" t="inlineStr">
         <is>
           <t>Naukri Direct NVite</t>
         </is>
       </c>
-      <c r="K91" s="20" t="inlineStr">
+      <c r="K91" s="15" t="inlineStr">
         <is>
           <t>Evaluated Recex Data Architect role. Requisition requires mandatory B.Tech/BE Computer Science, heavy Databricks/Spark/Scala coding, and CI/CD DevOps. Skipped per candidate rule.</t>
         </is>
       </c>
-      <c r="L91" s="20" t="inlineStr">
+      <c r="L91" s="15" t="inlineStr">
         <is>
           <t>2026-08-12</t>
         </is>
       </c>
-      <c r="M91" s="20" t="inlineStr">
+      <c r="M91" s="15" t="inlineStr">
         <is>
           <t>Target 14-20 LPA</t>
         </is>
       </c>
-      <c r="N91" s="20" t="inlineStr">
+      <c r="N91" s="15" t="inlineStr">
         <is>
           <t>Skipped Recex Data Architect role due to strict BE/BTech CS degree requirement and heavy Spark/Scala coding asks.</t>
         </is>
       </c>
-      <c r="O91" s="20" t="inlineStr">
+      <c r="O91" s="15" t="inlineStr">
         <is>
           <t>Reviewed - Deprioritized</t>
         </is>
       </c>
     </row>
-    <row r="92" ht="33.95" customHeight="1" s="17">
-      <c r="A92" s="20" t="inlineStr">
+    <row r="92" ht="33.95" customHeight="1" s="20">
+      <c r="A92" s="15" t="inlineStr">
         <is>
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="B92" s="20" t="inlineStr">
+      <c r="B92" s="15" t="inlineStr">
         <is>
           <t>IT Services &amp; Consulting Client (Naukri NVite)</t>
         </is>
       </c>
-      <c r="C92" s="20" t="inlineStr">
+      <c r="C92" s="15" t="inlineStr">
         <is>
           <t>Lead Power BI Developer / Senior Power BI Developer</t>
         </is>
       </c>
-      <c r="D92" s="20" t="inlineStr">
+      <c r="D92" s="15" t="inlineStr">
         <is>
           <t>Hyderabad / Remote</t>
         </is>
       </c>
-      <c r="E92" s="20" t="inlineStr">
+      <c r="E92" s="15" t="inlineStr">
         <is>
           <t>Naukri Recruiter Direct NVite</t>
         </is>
       </c>
-      <c r="F92" s="20" t="n">
+      <c r="F92" s="27" t="n">
         <v>0.98</v>
       </c>
-      <c r="G92" s="20" t="inlineStr">
-        <is>
-          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
-        </is>
-      </c>
-      <c r="H92" s="20" t="inlineStr">
+      <c r="G92" s="15" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H92" s="15" t="inlineStr">
         <is>
           <t>NVite Accepted &amp; Applied (7.0 - 17.0 LPA)</t>
         </is>
       </c>
-      <c r="I92" s="20" t="inlineStr">
+      <c r="I92" s="15" t="inlineStr">
         <is>
           <t>Recruiter NVite Team</t>
         </is>
       </c>
-      <c r="J92" s="20" t="inlineStr">
+      <c r="J92" s="15" t="inlineStr">
         <is>
           <t>Naukri Direct NVite</t>
         </is>
       </c>
-      <c r="K92" s="20" t="inlineStr">
+      <c r="K92" s="15" t="inlineStr">
         <is>
           <t>100% Core Skill Match. Requirements: Power BI, Senior Power BI Developer, Lead BI Developer, DAX, SQL. Salary: 7.0 - 17.0 LPA.</t>
         </is>
       </c>
-      <c r="L92" s="20" t="inlineStr">
+      <c r="L92" s="15" t="inlineStr">
         <is>
           <t>2026-08-12</t>
         </is>
       </c>
-      <c r="M92" s="20" t="inlineStr">
+      <c r="M92" s="15" t="inlineStr">
         <is>
           <t>7.0 - 17.0 LPA</t>
         </is>
       </c>
-      <c r="N92" s="20" t="inlineStr">
+      <c r="N92" s="15" t="inlineStr">
         <is>
           <t>Direct Recruiter NVite on Naukri for Lead / Senior Power BI Developer (7.0 - 17.0 LPA). 100% skill match.</t>
         </is>
       </c>
-      <c r="O92" s="20" t="inlineStr">
+      <c r="O92" s="15" t="inlineStr">
         <is>
           <t>Active - Target Applied</t>
         </is>
       </c>
     </row>
-    <row r="93" ht="33.95" customHeight="1" s="17">
-      <c r="A93" s="20" t="inlineStr">
+    <row r="93" ht="33.95" customHeight="1" s="20">
+      <c r="A93" s="15" t="inlineStr">
         <is>
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="B93" s="20" t="inlineStr">
+      <c r="B93" s="15" t="inlineStr">
         <is>
           <t>Nisvan HR Solutions (IT Client)</t>
         </is>
       </c>
-      <c r="C93" s="20" t="inlineStr">
+      <c r="C93" s="15" t="inlineStr">
         <is>
           <t>Snowflake Data Engineer (Tech Lead / Architect)</t>
         </is>
       </c>
-      <c r="D93" s="20" t="inlineStr">
+      <c r="D93" s="15" t="inlineStr">
         <is>
           <t>Bengaluru, Hyderabad, Pune</t>
         </is>
       </c>
-      <c r="E93" s="20" t="inlineStr">
+      <c r="E93" s="15" t="inlineStr">
         <is>
           <t>Naukri Recruiter Direct NVite</t>
         </is>
       </c>
-      <c r="F93" s="20" t="n">
+      <c r="F93" s="27" t="n">
         <v>0.99</v>
       </c>
-      <c r="G93" s="20" t="inlineStr">
-        <is>
-          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
-        </is>
-      </c>
-      <c r="H93" s="20" t="inlineStr">
+      <c r="G93" s="15" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H93" s="15" t="inlineStr">
         <is>
           <t>Application Submitted &amp; Confirmed (Naukri Direct - 22.5 to 25.0 LPA)</t>
         </is>
       </c>
-      <c r="I93" s="20" t="inlineStr">
+      <c r="I93" s="15" t="inlineStr">
         <is>
           <t>Nisvan HR Solutions Team</t>
         </is>
       </c>
-      <c r="J93" s="20" t="inlineStr">
+      <c r="J93" s="15" t="inlineStr">
         <is>
           <t>Naukri Direct NVite</t>
         </is>
       </c>
-      <c r="K93" s="20" t="inlineStr">
+      <c r="K93" s="15" t="inlineStr">
         <is>
           <t>Applied via Naukri for Nisvan HR Solutions Snowflake Data Engineer (22.5 - 25.0 LPA). Requirements: 10-12 Yrs Data Eng, 2+ Yrs Snowflake, Advanced SQL, Data Governance, Dimensional Modeling, Team Lead.</t>
         </is>
       </c>
-      <c r="L93" s="20" t="inlineStr">
+      <c r="L93" s="15" t="inlineStr">
         <is>
           <t>2026-08-12</t>
         </is>
       </c>
-      <c r="M93" s="20" t="inlineStr">
+      <c r="M93" s="15" t="inlineStr">
         <is>
           <t>22.5 - 25.0 LPA</t>
         </is>
       </c>
-      <c r="N93" s="20" t="inlineStr">
+      <c r="N93" s="15" t="inlineStr">
         <is>
           <t>Recruiter questionnaire completed and application officially submitted on Naukri for Nisvan HR Solutions Snowflake Data Engineer (22.5 - 25.0 LPA).</t>
         </is>
       </c>
-      <c r="O93" s="20" t="inlineStr">
+      <c r="O93" s="15" t="inlineStr">
         <is>
           <t>Active - Target Applied</t>
         </is>
       </c>
     </row>
-    <row r="94" ht="33.95" customHeight="1" s="17">
-      <c r="A94" s="20" t="inlineStr">
+    <row r="94" ht="33.95" customHeight="1" s="20">
+      <c r="A94" s="15" t="inlineStr">
         <is>
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="B94" s="20" t="inlineStr">
+      <c r="B94" s="15" t="inlineStr">
         <is>
           <t>IT Services &amp; Consulting Client (Naukri NVite)</t>
         </is>
       </c>
-      <c r="C94" s="20" t="inlineStr">
+      <c r="C94" s="15" t="inlineStr">
         <is>
           <t>Data Engineering Lead</t>
         </is>
       </c>
-      <c r="D94" s="20" t="inlineStr">
+      <c r="D94" s="15" t="inlineStr">
         <is>
           <t>Hyderabad, Thiruvananthapuram, Noida</t>
         </is>
       </c>
-      <c r="E94" s="20" t="inlineStr">
+      <c r="E94" s="15" t="inlineStr">
         <is>
           <t>Naukri Recruiter Direct NVite</t>
         </is>
       </c>
-      <c r="F94" s="20" t="n">
+      <c r="F94" s="27" t="n">
         <v>0.98</v>
       </c>
-      <c r="G94" s="20" t="inlineStr">
-        <is>
-          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
-        </is>
-      </c>
-      <c r="H94" s="20" t="inlineStr">
+      <c r="G94" s="15" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H94" s="15" t="inlineStr">
         <is>
           <t>NVite Accepted &amp; Applied</t>
         </is>
       </c>
-      <c r="I94" s="20" t="inlineStr">
+      <c r="I94" s="15" t="inlineStr">
         <is>
           <t>Naukri Recruiter Direct</t>
         </is>
       </c>
-      <c r="J94" s="20" t="inlineStr">
+      <c r="J94" s="15" t="inlineStr">
         <is>
           <t>Naukri Direct NVite</t>
         </is>
       </c>
-      <c r="K94" s="20" t="inlineStr">
+      <c r="K94" s="15" t="inlineStr">
         <is>
           <t>98% Skill Match for Data Engineering Lead. Requirements: ETL, SQL, Data Governance &amp; Pipeline Management.</t>
         </is>
       </c>
-      <c r="L94" s="20" t="inlineStr">
+      <c r="L94" s="15" t="inlineStr">
         <is>
           <t>2026-08-12</t>
         </is>
       </c>
-      <c r="M94" s="20" t="inlineStr">
+      <c r="M94" s="15" t="inlineStr">
         <is>
           <t>Not Disclosed / High Senior Package</t>
         </is>
       </c>
-      <c r="N94" s="20" t="inlineStr">
+      <c r="N94" s="15" t="inlineStr">
         <is>
           <t>Direct Recruiter NVite on Naukri for Data Engineering Lead (2h ago). NVite accepted &amp; applied.</t>
         </is>
       </c>
-      <c r="O94" s="20" t="inlineStr">
+      <c r="O94" s="15" t="inlineStr">
         <is>
           <t>Active - Target Applied</t>
         </is>
       </c>
     </row>
-    <row r="95" ht="33.95" customHeight="1" s="17">
-      <c r="A95" s="20" t="inlineStr">
+    <row r="95" ht="33.95" customHeight="1" s="20">
+      <c r="A95" s="15" t="inlineStr">
         <is>
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="B95" s="20" t="inlineStr">
+      <c r="B95" s="15" t="inlineStr">
         <is>
           <t>Pyramid IT Consulting</t>
         </is>
       </c>
-      <c r="C95" s="20" t="inlineStr">
+      <c r="C95" s="15" t="inlineStr">
         <is>
           <t>Senior Data / IT Role (Naukri NVite)</t>
         </is>
       </c>
-      <c r="D95" s="20" t="inlineStr">
+      <c r="D95" s="15" t="inlineStr">
         <is>
           <t>NOIDA / Remote</t>
         </is>
       </c>
-      <c r="E95" s="20" t="inlineStr">
+      <c r="E95" s="15" t="inlineStr">
         <is>
           <t>Naukri Recruiter Direct NVite</t>
         </is>
       </c>
-      <c r="F95" s="20" t="n">
+      <c r="F95" s="27" t="n">
         <v>0.95</v>
       </c>
-      <c r="G95" s="20" t="inlineStr">
-        <is>
-          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
-        </is>
-      </c>
-      <c r="H95" s="20" t="inlineStr">
+      <c r="G95" s="15" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H95" s="15" t="inlineStr">
         <is>
           <t>NVite Received (Accepted &amp; Profile Connected)</t>
         </is>
       </c>
-      <c r="I95" s="20" t="inlineStr">
+      <c r="I95" s="15" t="inlineStr">
         <is>
           <t>Ankit Kumar (VP at Pyramid IT Consulting)</t>
         </is>
       </c>
-      <c r="J95" s="20" t="inlineStr">
+      <c r="J95" s="15" t="inlineStr">
         <is>
           <t>Noida Direct NVite</t>
         </is>
       </c>
-      <c r="K95" s="20" t="inlineStr">
+      <c r="K95" s="15" t="inlineStr">
         <is>
           <t>NVite received from VP level recruiter (Ankit Kumar, VP at Pyramid IT Consulting). NVite accepted on Naukri.</t>
         </is>
       </c>
-      <c r="L95" s="20" t="inlineStr">
+      <c r="L95" s="15" t="inlineStr">
         <is>
           <t>2026-08-12</t>
         </is>
       </c>
-      <c r="M95" s="20" t="inlineStr">
+      <c r="M95" s="15" t="inlineStr">
         <is>
           <t>Not Disclosed / Senior CTC Band</t>
         </is>
       </c>
-      <c r="N95" s="20" t="inlineStr">
+      <c r="N95" s="15" t="inlineStr">
         <is>
           <t>VP level outreach from Pyramid IT Consulting (Ankit Kumar, VP). NVite accepted on Naukri.</t>
         </is>
       </c>
-      <c r="O95" s="20" t="inlineStr">
+      <c r="O95" s="15" t="inlineStr">
         <is>
           <t>Active - Target Applied</t>
         </is>
       </c>
     </row>
-    <row r="96" ht="33.95" customHeight="1" s="17"/>
-    <row r="97" ht="33.95" customHeight="1" s="17"/>
-    <row r="98" ht="33.95" customHeight="1" s="17"/>
-    <row r="99" ht="33.95" customHeight="1" s="17"/>
-    <row r="100" ht="33.95" customHeight="1" s="17"/>
-    <row r="101" ht="33.95" customHeight="1" s="17"/>
-    <row r="102" ht="33.95" customHeight="1" s="17"/>
-    <row r="103" ht="33.95" customHeight="1" s="17"/>
-    <row r="104" ht="33.95" customHeight="1" s="17"/>
-    <row r="105" ht="33.95" customHeight="1" s="17"/>
-    <row r="106" ht="33.95" customHeight="1" s="17"/>
-    <row r="107" ht="33.95" customHeight="1" s="17"/>
-    <row r="108" ht="33.95" customHeight="1" s="17"/>
-    <row r="109" ht="33.95" customHeight="1" s="17"/>
-    <row r="110" ht="33.95" customHeight="1" s="17"/>
-    <row r="111" ht="33.95" customHeight="1" s="17"/>
-    <row r="112" ht="33.95" customHeight="1" s="17"/>
-    <row r="113" ht="33.95" customHeight="1" s="17"/>
-    <row r="114" ht="33.95" customHeight="1" s="17"/>
-    <row r="115" ht="33.95" customHeight="1" s="17"/>
-    <row r="116" ht="33.95" customHeight="1" s="17"/>
-    <row r="117" ht="33.95" customHeight="1" s="17"/>
-    <row r="118" ht="33.95" customHeight="1" s="17"/>
-    <row r="119" ht="33.95" customHeight="1" s="17"/>
-    <row r="120" ht="33.95" customHeight="1" s="17"/>
-    <row r="121" ht="33.95" customHeight="1" s="17"/>
-    <row r="122" ht="33.95" customHeight="1" s="17"/>
-    <row r="123" ht="33.95" customHeight="1" s="17"/>
-    <row r="124" ht="33.95" customHeight="1" s="17"/>
-    <row r="125" ht="33.95" customHeight="1" s="17"/>
-    <row r="126" ht="33.95" customHeight="1" s="17"/>
-    <row r="127" ht="33.95" customHeight="1" s="17"/>
-    <row r="128" ht="33.95" customHeight="1" s="17"/>
-    <row r="129" ht="33.95" customHeight="1" s="17"/>
-    <row r="130" ht="33.95" customHeight="1" s="17"/>
-    <row r="131" ht="33.95" customHeight="1" s="17"/>
-    <row r="132" ht="33.95" customHeight="1" s="17"/>
-    <row r="133" ht="33.95" customHeight="1" s="17"/>
-    <row r="134" ht="33.95" customHeight="1" s="17"/>
-    <row r="135" ht="33.95" customHeight="1" s="17"/>
-    <row r="136" ht="33.95" customHeight="1" s="17"/>
-    <row r="137" ht="33.95" customHeight="1" s="17"/>
-    <row r="138" ht="33.95" customHeight="1" s="17"/>
-    <row r="139" ht="33.95" customHeight="1" s="17"/>
-    <row r="140" ht="33.95" customHeight="1" s="17"/>
-    <row r="141" ht="33.95" customHeight="1" s="17"/>
-    <row r="142" ht="33.95" customHeight="1" s="17"/>
-    <row r="143" ht="33.95" customHeight="1" s="17"/>
-    <row r="144" ht="33.95" customHeight="1" s="17"/>
-    <row r="145" ht="33.95" customHeight="1" s="17"/>
-    <row r="146" ht="33.95" customHeight="1" s="17"/>
-    <row r="147" ht="33.95" customHeight="1" s="17"/>
-    <row r="148" ht="33.95" customHeight="1" s="17"/>
-    <row r="149" ht="33.95" customHeight="1" s="17"/>
-    <row r="150" ht="33.95" customHeight="1" s="17"/>
-    <row r="151" ht="33.95" customHeight="1" s="17"/>
-    <row r="152" ht="33.95" customHeight="1" s="17"/>
-    <row r="153" ht="33.95" customHeight="1" s="17"/>
-    <row r="154" ht="33.95" customHeight="1" s="17"/>
-    <row r="155" ht="33.95" customHeight="1" s="17"/>
-    <row r="156" ht="33.95" customHeight="1" s="17"/>
-    <row r="157" ht="33.95" customHeight="1" s="17"/>
-    <row r="158" ht="33.95" customHeight="1" s="17"/>
-    <row r="159" ht="33.95" customHeight="1" s="17"/>
-    <row r="160" ht="33.95" customHeight="1" s="17"/>
-    <row r="161" ht="33.95" customHeight="1" s="17"/>
-    <row r="162" ht="33.95" customHeight="1" s="17"/>
-    <row r="163" ht="33.95" customHeight="1" s="17"/>
-    <row r="164" ht="33.95" customHeight="1" s="17"/>
-    <row r="165" ht="33.95" customHeight="1" s="17"/>
-    <row r="166" ht="33.95" customHeight="1" s="17"/>
-    <row r="167" ht="33.95" customHeight="1" s="17"/>
-    <row r="168" ht="33.95" customHeight="1" s="17"/>
-    <row r="169" ht="33.95" customHeight="1" s="17"/>
-    <row r="170" ht="33.95" customHeight="1" s="17"/>
-    <row r="171" ht="33.95" customHeight="1" s="17"/>
-    <row r="172" ht="33.95" customHeight="1" s="17"/>
-    <row r="173" ht="33.95" customHeight="1" s="17"/>
-    <row r="174" ht="33.95" customHeight="1" s="17"/>
-    <row r="175" ht="33.95" customHeight="1" s="17"/>
-    <row r="176" ht="33.95" customHeight="1" s="17"/>
-    <row r="177" ht="33.95" customHeight="1" s="17"/>
-    <row r="178" ht="33.95" customHeight="1" s="17"/>
-    <row r="179" ht="33.95" customHeight="1" s="17"/>
-    <row r="180" ht="33.95" customHeight="1" s="17"/>
-    <row r="181" ht="33.95" customHeight="1" s="17"/>
-    <row r="182" ht="33.95" customHeight="1" s="17"/>
-    <row r="183" ht="33.95" customHeight="1" s="17"/>
-    <row r="184" ht="33.95" customHeight="1" s="17"/>
-    <row r="185" ht="33.95" customHeight="1" s="17"/>
-    <row r="186" ht="33.95" customHeight="1" s="17"/>
-    <row r="187" ht="33.95" customHeight="1" s="17"/>
-    <row r="188" ht="33.95" customHeight="1" s="17"/>
-    <row r="189" ht="33.95" customHeight="1" s="17"/>
-    <row r="190" ht="33.95" customHeight="1" s="17"/>
-    <row r="191" ht="33.95" customHeight="1" s="17"/>
-    <row r="192" ht="33.95" customHeight="1" s="17"/>
-    <row r="193" ht="33.95" customHeight="1" s="17"/>
-    <row r="194" ht="33.95" customHeight="1" s="17"/>
-    <row r="195" ht="33.95" customHeight="1" s="17"/>
-    <row r="196" ht="33.95" customHeight="1" s="17"/>
-    <row r="197" ht="33.95" customHeight="1" s="17"/>
-    <row r="198" ht="33.95" customHeight="1" s="17"/>
-    <row r="199" ht="33.95" customHeight="1" s="17"/>
-    <row r="200" ht="33.95" customHeight="1" s="17"/>
-    <row r="201" ht="33.95" customHeight="1" s="17"/>
-    <row r="202" ht="33.95" customHeight="1" s="17"/>
-    <row r="203" ht="33.95" customHeight="1" s="17"/>
-    <row r="204" ht="33.95" customHeight="1" s="17"/>
-    <row r="205" ht="33.95" customHeight="1" s="17"/>
+    <row r="96" ht="33.95" customHeight="1" s="20">
+      <c r="A96" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B96" s="29" t="inlineStr">
+        <is>
+          <t>Growel Softech Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="C96" s="29" t="inlineStr">
+        <is>
+          <t>Snowflake Data Engineer</t>
+        </is>
+      </c>
+      <c r="D96" s="29" t="inlineStr">
+        <is>
+          <t>Bengaluru (In Office)</t>
+        </is>
+      </c>
+      <c r="E96" s="29" t="inlineStr">
+        <is>
+          <t>Naukri Recruiter Direct NVite</t>
+        </is>
+      </c>
+      <c r="F96" s="29" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="G96" s="29" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H96" s="29" t="inlineStr">
+        <is>
+          <t>Application Submitted &amp; Confirmed (0 - 15.0 LPA)</t>
+        </is>
+      </c>
+      <c r="I96" s="29" t="inlineStr">
+        <is>
+          <t>Growel Softech TA Team</t>
+        </is>
+      </c>
+      <c r="J96" s="29" t="inlineStr">
+        <is>
+          <t>Naukri Direct NVite</t>
+        </is>
+      </c>
+      <c r="K96" s="29" t="inlineStr">
+        <is>
+          <t>98% Skill Match for Snowflake &amp; Data Engineering. Explicit requirement: Graduation Not Required. Applied Aug 11.</t>
+        </is>
+      </c>
+      <c r="L96" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M96" s="29" t="inlineStr">
+        <is>
+          <t>0 - 15.0 LPA</t>
+        </is>
+      </c>
+      <c r="N96" s="29" t="inlineStr">
+        <is>
+          <t>Applied on Naukri for Growel Softech Snowflake Data Engineer. Explicitly specifies Graduation Not Required.</t>
+        </is>
+      </c>
+      <c r="O96" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="33.95" customHeight="1" s="20">
+      <c r="A97" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B97" s="29" t="inlineStr">
+        <is>
+          <t>Growel Softech Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="C97" s="29" t="inlineStr">
+        <is>
+          <t>Snowflake Data Engineer (dbt &amp; SQL)</t>
+        </is>
+      </c>
+      <c r="D97" s="29" t="inlineStr">
+        <is>
+          <t>Hyderabad, Chennai, Bengaluru (Hybrid)</t>
+        </is>
+      </c>
+      <c r="E97" s="29" t="inlineStr">
+        <is>
+          <t>Naukri Recruiter Direct NVite</t>
+        </is>
+      </c>
+      <c r="F97" s="29" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G97" s="29" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H97" s="29" t="inlineStr">
+        <is>
+          <t>Application Submitted &amp; Confirmed (Naukri NVite)</t>
+        </is>
+      </c>
+      <c r="I97" s="29" t="inlineStr">
+        <is>
+          <t>Growel Softech TA Team</t>
+        </is>
+      </c>
+      <c r="J97" s="29" t="inlineStr">
+        <is>
+          <t>Naukri Direct NVite</t>
+        </is>
+      </c>
+      <c r="K97" s="29" t="inlineStr">
+        <is>
+          <t>99% Skill Match. Primary: SQL + Snowflake, Secondary: dbt. 10-14 Yrs Exp. Customer Round Yes.</t>
+        </is>
+      </c>
+      <c r="L97" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M97" s="29" t="inlineStr">
+        <is>
+          <t>Not Disclosed / High Senior Band</t>
+        </is>
+      </c>
+      <c r="N97" s="29" t="inlineStr">
+        <is>
+          <t>Application officially submitted on Naukri for Growel Softech Snowflake Data Engineer (dbt &amp; SQL). Core skills match 100% (Snowflake Accredible Badge &amp; dbt in master resume).</t>
+        </is>
+      </c>
+      <c r="O97" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="33.95" customHeight="1" s="20"/>
+    <row r="99" ht="33.95" customHeight="1" s="20"/>
+    <row r="100" ht="33.95" customHeight="1" s="20"/>
+    <row r="101" ht="33.95" customHeight="1" s="20"/>
+    <row r="102" ht="33.95" customHeight="1" s="20"/>
+    <row r="103" ht="33.95" customHeight="1" s="20"/>
+    <row r="104" ht="33.95" customHeight="1" s="20"/>
+    <row r="105" ht="33.95" customHeight="1" s="20"/>
+    <row r="106" ht="33.95" customHeight="1" s="20"/>
+    <row r="107" ht="33.95" customHeight="1" s="20"/>
+    <row r="108" ht="33.95" customHeight="1" s="20"/>
+    <row r="109" ht="33.95" customHeight="1" s="20"/>
+    <row r="110" ht="33.95" customHeight="1" s="20"/>
+    <row r="111" ht="33.95" customHeight="1" s="20"/>
+    <row r="112" ht="33.95" customHeight="1" s="20"/>
+    <row r="113" ht="33.95" customHeight="1" s="20"/>
+    <row r="114" ht="33.95" customHeight="1" s="20"/>
+    <row r="115" ht="33.95" customHeight="1" s="20"/>
+    <row r="116" ht="33.95" customHeight="1" s="20"/>
+    <row r="117" ht="33.95" customHeight="1" s="20"/>
+    <row r="118" ht="33.95" customHeight="1" s="20"/>
+    <row r="119" ht="33.95" customHeight="1" s="20"/>
+    <row r="120" ht="33.95" customHeight="1" s="20"/>
+    <row r="121" ht="33.95" customHeight="1" s="20"/>
+    <row r="122" ht="33.95" customHeight="1" s="20"/>
+    <row r="123" ht="33.95" customHeight="1" s="20"/>
+    <row r="124" ht="33.95" customHeight="1" s="20"/>
+    <row r="125" ht="33.95" customHeight="1" s="20"/>
+    <row r="126" ht="33.95" customHeight="1" s="20"/>
+    <row r="127" ht="33.95" customHeight="1" s="20"/>
+    <row r="128" ht="33.95" customHeight="1" s="20"/>
+    <row r="129" ht="33.95" customHeight="1" s="20"/>
+    <row r="130" ht="33.95" customHeight="1" s="20"/>
+    <row r="131" ht="33.95" customHeight="1" s="20"/>
+    <row r="132" ht="33.95" customHeight="1" s="20"/>
+    <row r="133" ht="33.95" customHeight="1" s="20"/>
+    <row r="134" ht="33.95" customHeight="1" s="20"/>
+    <row r="135" ht="33.95" customHeight="1" s="20"/>
+    <row r="136" ht="33.95" customHeight="1" s="20"/>
+    <row r="137" ht="33.95" customHeight="1" s="20"/>
+    <row r="138" ht="33.95" customHeight="1" s="20"/>
+    <row r="139" ht="33.95" customHeight="1" s="20"/>
+    <row r="140" ht="33.95" customHeight="1" s="20"/>
+    <row r="141" ht="33.95" customHeight="1" s="20"/>
+    <row r="142" ht="33.95" customHeight="1" s="20"/>
+    <row r="143" ht="33.95" customHeight="1" s="20"/>
+    <row r="144" ht="33.95" customHeight="1" s="20"/>
+    <row r="145" ht="33.95" customHeight="1" s="20"/>
+    <row r="146" ht="33.95" customHeight="1" s="20"/>
+    <row r="147" ht="33.95" customHeight="1" s="20"/>
+    <row r="148" ht="33.95" customHeight="1" s="20"/>
+    <row r="149" ht="33.95" customHeight="1" s="20"/>
+    <row r="150" ht="33.95" customHeight="1" s="20"/>
+    <row r="151" ht="33.95" customHeight="1" s="20"/>
+    <row r="152" ht="33.95" customHeight="1" s="20"/>
+    <row r="153" ht="33.95" customHeight="1" s="20"/>
+    <row r="154" ht="33.95" customHeight="1" s="20"/>
+    <row r="155" ht="33.95" customHeight="1" s="20"/>
+    <row r="156" ht="33.95" customHeight="1" s="20"/>
+    <row r="157" ht="33.95" customHeight="1" s="20"/>
+    <row r="158" ht="33.95" customHeight="1" s="20"/>
+    <row r="159" ht="33.95" customHeight="1" s="20"/>
+    <row r="160" ht="33.95" customHeight="1" s="20"/>
+    <row r="161" ht="33.95" customHeight="1" s="20"/>
+    <row r="162" ht="33.95" customHeight="1" s="20"/>
+    <row r="163" ht="33.95" customHeight="1" s="20"/>
+    <row r="164" ht="33.95" customHeight="1" s="20"/>
+    <row r="165" ht="33.95" customHeight="1" s="20"/>
+    <row r="166" ht="33.95" customHeight="1" s="20"/>
+    <row r="167" ht="33.95" customHeight="1" s="20"/>
+    <row r="168" ht="33.95" customHeight="1" s="20"/>
+    <row r="169" ht="33.95" customHeight="1" s="20"/>
+    <row r="170" ht="33.95" customHeight="1" s="20"/>
+    <row r="171" ht="33.95" customHeight="1" s="20"/>
+    <row r="172" ht="33.95" customHeight="1" s="20"/>
+    <row r="173" ht="33.95" customHeight="1" s="20"/>
+    <row r="174" ht="33.95" customHeight="1" s="20"/>
+    <row r="175" ht="33.95" customHeight="1" s="20"/>
+    <row r="176" ht="33.95" customHeight="1" s="20"/>
+    <row r="177" ht="33.95" customHeight="1" s="20"/>
+    <row r="178" ht="33.95" customHeight="1" s="20"/>
+    <row r="179" ht="33.95" customHeight="1" s="20"/>
+    <row r="180" ht="33.95" customHeight="1" s="20"/>
+    <row r="181" ht="33.95" customHeight="1" s="20"/>
+    <row r="182" ht="33.95" customHeight="1" s="20"/>
+    <row r="183" ht="33.95" customHeight="1" s="20"/>
+    <row r="184" ht="33.95" customHeight="1" s="20"/>
+    <row r="185" ht="33.95" customHeight="1" s="20"/>
+    <row r="186" ht="33.95" customHeight="1" s="20"/>
+    <row r="187" ht="33.95" customHeight="1" s="20"/>
+    <row r="188" ht="33.95" customHeight="1" s="20"/>
+    <row r="189" ht="33.95" customHeight="1" s="20"/>
+    <row r="190" ht="33.95" customHeight="1" s="20"/>
+    <row r="191" ht="33.95" customHeight="1" s="20"/>
+    <row r="192" ht="33.95" customHeight="1" s="20"/>
+    <row r="193" ht="33.95" customHeight="1" s="20"/>
+    <row r="194" ht="33.95" customHeight="1" s="20"/>
+    <row r="195" ht="33.95" customHeight="1" s="20"/>
+    <row r="196" ht="33.95" customHeight="1" s="20"/>
+    <row r="197" ht="33.95" customHeight="1" s="20"/>
+    <row r="198" ht="33.95" customHeight="1" s="20"/>
+    <row r="199" ht="33.95" customHeight="1" s="20"/>
+    <row r="200" ht="33.95" customHeight="1" s="20"/>
+    <row r="201" ht="33.95" customHeight="1" s="20"/>
+    <row r="202" ht="33.95" customHeight="1" s="20"/>
+    <row r="203" ht="33.95" customHeight="1" s="20"/>
+    <row r="204" ht="33.95" customHeight="1" s="20"/>
+    <row r="205" ht="33.95" customHeight="1" s="20"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:O1"/>
@@ -7013,10 +7181,10 @@
   <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
-    <col width="24" customWidth="1" style="17" min="1" max="3"/>
+    <col width="24" customWidth="1" style="20" min="1" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" s="17">
+    <row r="1" ht="15" customHeight="1" s="20">
       <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Application Status</t>
@@ -7189,18 +7357,18 @@
   <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
-    <col width="8" customWidth="1" style="17" min="1" max="1"/>
-    <col width="85" customWidth="1" style="17" min="2" max="2"/>
+    <col width="8" customWidth="1" style="20" min="1" max="1"/>
+    <col width="85" customWidth="1" style="20" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="27.95" customHeight="1" s="17">
-      <c r="A1" s="19" t="inlineStr">
+    <row r="1" ht="27.95" customHeight="1" s="20">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>How to Use This Tracker</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="26.1" customHeight="1" s="17">
+    <row r="3" ht="26.1" customHeight="1" s="20">
       <c r="A3" s="4" t="inlineStr">
         <is>
           <t>1</t>
@@ -7212,7 +7380,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="26.1" customHeight="1" s="17">
+    <row r="4" ht="26.1" customHeight="1" s="20">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>2</t>
@@ -7224,7 +7392,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="26.1" customHeight="1" s="17">
+    <row r="5" ht="26.1" customHeight="1" s="20">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>3</t>
@@ -7236,7 +7404,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="26.1" customHeight="1" s="17">
+    <row r="6" ht="26.1" customHeight="1" s="20">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>4</t>
@@ -7248,7 +7416,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="26.1" customHeight="1" s="17">
+    <row r="7" ht="26.1" customHeight="1" s="20">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>5</t>

</xml_diff>

<commit_message>
Tuesday Aug 11: Logged Innova ESI Data Analytics (Bangalore) opportunity in tracker Row 98
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -226,7 +226,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -289,6 +289,9 @@
     <xf numFmtId="9" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -722,7 +725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O97"/>
+  <dimension ref="A1:O98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -2309,15 +2312,19 @@
           <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
         </is>
       </c>
-      <c r="H27" s="8" t="inlineStr">
-        <is>
-          <t>Submitted</t>
-        </is>
-      </c>
-      <c r="I27" s="7" t="n"/>
+      <c r="H27" s="30" t="inlineStr">
+        <is>
+          <t>Naukri Profile Viewed by India Head (naukri7 - LanceSoft)</t>
+        </is>
+      </c>
+      <c r="I27" s="7" t="inlineStr">
+        <is>
+          <t>naukri7 (India Head at LanceSoft)</t>
+        </is>
+      </c>
       <c r="J27" s="7" t="inlineStr">
         <is>
-          <t>hr.dinesh06@gmail.com</t>
+          <t>Bangalore Direct View</t>
         </is>
       </c>
       <c r="K27" s="7" t="inlineStr">
@@ -2333,7 +2340,7 @@
       </c>
       <c r="N27" s="7" t="inlineStr">
         <is>
-          <t>Recruiter Outreach. Profile viewed on Naukri. Direct Email &amp; Resume sent to Dinesh Kumaar (`hr.dinesh06@gmail.com`).</t>
+          <t>Naukri Profile Viewed by India Head at LanceSoft (Bangalore) 1 hour ago. Active senior executive engagement.</t>
         </is>
       </c>
       <c r="O27" s="6" t="inlineStr">
@@ -6686,12 +6693,12 @@
       </c>
       <c r="I93" s="15" t="inlineStr">
         <is>
-          <t>Nisvan HR Solutions Team</t>
+          <t>Kavita Bansal (Director at Nisvan HR Solutions)</t>
         </is>
       </c>
       <c r="J93" s="15" t="inlineStr">
         <is>
-          <t>Naukri Direct NVite</t>
+          <t>Mohali Direct NVite</t>
         </is>
       </c>
       <c r="K93" s="15" t="inlineStr">
@@ -6911,7 +6918,7 @@
       </c>
       <c r="I96" s="29" t="inlineStr">
         <is>
-          <t>Growel Softech TA Team</t>
+          <t>Snehal Hegu (Sr Recruiter at Growel Softech)</t>
         </is>
       </c>
       <c r="J96" s="29" t="inlineStr">
@@ -6986,7 +6993,7 @@
       </c>
       <c r="I97" s="29" t="inlineStr">
         <is>
-          <t>Growel Softech TA Team</t>
+          <t>Snehal Hegu (Sr Recruiter at Growel Softech)</t>
         </is>
       </c>
       <c r="J97" s="29" t="inlineStr">
@@ -7020,7 +7027,81 @@
         </is>
       </c>
     </row>
-    <row r="98" ht="33.95" customHeight="1" s="20"/>
+    <row r="98" ht="33.95" customHeight="1" s="20">
+      <c r="A98" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B98" s="29" t="inlineStr">
+        <is>
+          <t>Innova ESI</t>
+        </is>
+      </c>
+      <c r="C98" s="29" t="inlineStr">
+        <is>
+          <t>Data Analytics Professional (Azure, SQL &amp; Power BI)</t>
+        </is>
+      </c>
+      <c r="D98" s="29" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="E98" s="29" t="inlineStr">
+        <is>
+          <t>LinkedIn Direct (connect@innovaesi.com)</t>
+        </is>
+      </c>
+      <c r="F98" s="29" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="G98" s="29" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H98" s="29" t="inlineStr">
+        <is>
+          <t>Target Opportunity Logged (Email + Web Form)</t>
+        </is>
+      </c>
+      <c r="I98" s="29" t="inlineStr">
+        <is>
+          <t>Innova ESI Hiring Team</t>
+        </is>
+      </c>
+      <c r="J98" s="29" t="inlineStr">
+        <is>
+          <t>connect@innovaesi.com</t>
+        </is>
+      </c>
+      <c r="K98" s="29" t="inlineStr">
+        <is>
+          <t>98% Skill Match for Azure, SQL &amp; Power BI. Requirements: 3-6 Yrs, Azure SQL, Synapse, Power BI, SQL. Location: Bangalore.</t>
+        </is>
+      </c>
+      <c r="L98" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M98" s="29" t="inlineStr">
+        <is>
+          <t>Not Disclosed / Senior Band</t>
+        </is>
+      </c>
+      <c r="N98" s="29" t="inlineStr">
+        <is>
+          <t>Direct LinkedIn post from Innova ESI for Data Analytics (Bangalore). Email: connect@innovaesi.com | Web: https://lnkd.in/dGGdDVJi</t>
+        </is>
+      </c>
+      <c r="O98" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
     <row r="99" ht="33.95" customHeight="1" s="20"/>
     <row r="100" ht="33.95" customHeight="1" s="20"/>
     <row r="101" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Tuesday Aug 11: Follow-up email sent to Nandita Sharma (Mphasis HR) for Aug 6 & Aug 10 evaluation feedback
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -870,9 +870,9 @@
           <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
         </is>
       </c>
-      <c r="H5" s="17" t="inlineStr">
-        <is>
-          <t>L1 Senior Technical Interview Completed &amp; Rated (Risebird)</t>
+      <c r="H5" s="30" t="inlineStr">
+        <is>
+          <t>Follow-up Email Sent to HR (Nandita Sharma)</t>
         </is>
       </c>
       <c r="I5" s="7" t="inlineStr">
@@ -892,7 +892,7 @@
       </c>
       <c r="L5" s="6" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="M5" s="7" t="inlineStr">
@@ -902,7 +902,7 @@
       </c>
       <c r="N5" s="7" t="inlineStr">
         <is>
-          <t>Official candidate feedback submitted and confirmed on Risebird portal for Aug 10 Senior L1 interview.</t>
+          <t>Follow-up email sent on Tuesday Aug 11 to Nandita Sharma (nandita.sharma@mphasis.com) requesting consolidated feedback for Aug 6 &amp; Aug 10 L1 technical interviews and Stage 2 schedule.</t>
         </is>
       </c>
       <c r="O5" s="6" t="inlineStr">
@@ -7063,7 +7063,7 @@
       </c>
       <c r="H98" s="29" t="inlineStr">
         <is>
-          <t>Target Opportunity Logged (Email + Web Form)</t>
+          <t>Reviewed - Deprioritized (Low Response / Generic Post)</t>
         </is>
       </c>
       <c r="I98" s="29" t="inlineStr">
@@ -7093,7 +7093,7 @@
       </c>
       <c r="N98" s="29" t="inlineStr">
         <is>
-          <t>Direct LinkedIn post from Innova ESI for Data Analytics (Bangalore). Email: connect@innovaesi.com | Web: https://lnkd.in/dGGdDVJi</t>
+          <t>Deprioritized per candidate rule: Generic agency posting with zero direct HR response.</t>
         </is>
       </c>
       <c r="O98" s="29" t="inlineStr">

</xml_diff>

<commit_message>
Tuesday Aug 11: Logged UST Power BI Developer (Hyderabad) application in tracker Row 99
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -725,7 +725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O98"/>
+  <dimension ref="A1:O99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -1861,7 +1861,7 @@
       </c>
       <c r="H20" s="18" t="inlineStr">
         <is>
-          <t>Awaiting Calendar Slot Confirmation (Persistent Systems Stage 2)</t>
+          <t>Follow-up Sent on WhatsApp (Persistent Stage 2 Slot Pending)</t>
         </is>
       </c>
       <c r="I20" s="7" t="inlineStr">
@@ -1881,7 +1881,7 @@
       </c>
       <c r="L20" s="6" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="M20" s="7" t="inlineStr">
@@ -1891,7 +1891,7 @@
       </c>
       <c r="N20" s="7" t="inlineStr">
         <is>
-          <t>Pooja (Growel Softech) confirmed candidate shortlisted for Stage 2 Human Technical Round. Awaiting calendar invite/slot confirmation call from Persistent Systems.</t>
+          <t>WhatsApp follow-up sent on Monday Aug 10 @ 3:58 PM to Pooja (Growel HR 7992357043) requesting Persistent Systems Stage 2 slot confirmation.</t>
         </is>
       </c>
       <c r="O20" s="6" t="inlineStr">
@@ -7102,7 +7102,81 @@
         </is>
       </c>
     </row>
-    <row r="99" ht="33.95" customHeight="1" s="20"/>
+    <row r="99" ht="33.95" customHeight="1" s="20">
+      <c r="A99" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B99" s="29" t="inlineStr">
+        <is>
+          <t>UST (UST Global)</t>
+        </is>
+      </c>
+      <c r="C99" s="29" t="inlineStr">
+        <is>
+          <t>Power BI Developer (Enterprise Data Lead)</t>
+        </is>
+      </c>
+      <c r="D99" s="29" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana (On-site / Hybrid)</t>
+        </is>
+      </c>
+      <c r="E99" s="29" t="inlineStr">
+        <is>
+          <t>LinkedIn Direct Application</t>
+        </is>
+      </c>
+      <c r="F99" s="29" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G99" s="29" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H99" s="29" t="inlineStr">
+        <is>
+          <t>Application Submitted &amp; Confirmed (LinkedIn Direct)</t>
+        </is>
+      </c>
+      <c r="I99" s="29" t="inlineStr">
+        <is>
+          <t>UST Talent Acquisition / Jyothi Kondeti (Network)</t>
+        </is>
+      </c>
+      <c r="J99" s="29" t="inlineStr">
+        <is>
+          <t>LinkedIn Direct</t>
+        </is>
+      </c>
+      <c r="K99" s="29" t="inlineStr">
+        <is>
+          <t>99% Core Skill Match. Requirements: 6+ Yrs Power BI, DAX, Power Query M, Star Schema, Paginated Reports, RLS, Fabric, SQL Stored Procedures. Education: Bachelor or EQUIVALENT PRACTICAL EXPERIENCE.</t>
+        </is>
+      </c>
+      <c r="L99" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M99" s="29" t="inlineStr">
+        <is>
+          <t>Not Disclosed / Senior Enterprise Band</t>
+        </is>
+      </c>
+      <c r="N99" s="29" t="inlineStr">
+        <is>
+          <t>Direct LinkedIn application for UST Power BI Developer in Hyderabad. 99% match for Amazon Book Author &amp; 15 Yrs Data Lead. Explicitly accepts equivalent practical experience.</t>
+        </is>
+      </c>
+      <c r="O99" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
     <row r="100" ht="33.95" customHeight="1" s="20"/>
     <row r="101" ht="33.95" customHeight="1" s="20"/>
     <row r="102" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Tuesday Aug 11: Official application confirmed for UST Global Power BI Developer (Job ID: 620625 - Hyderabad)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -7138,7 +7138,7 @@
       </c>
       <c r="H99" s="29" t="inlineStr">
         <is>
-          <t>Application Submitted &amp; Confirmed (LinkedIn Direct)</t>
+          <t>Application Submitted &amp; Confirmed (Job ID: 620625)</t>
         </is>
       </c>
       <c r="I99" s="29" t="inlineStr">
@@ -7153,7 +7153,7 @@
       </c>
       <c r="K99" s="29" t="inlineStr">
         <is>
-          <t>99% Core Skill Match. Requirements: 6+ Yrs Power BI, DAX, Power Query M, Star Schema, Paginated Reports, RLS, Fabric, SQL Stored Procedures. Education: Bachelor or EQUIVALENT PRACTICAL EXPERIENCE.</t>
+          <t>Job ID: 620625 | 7 Years Exp | 1 Opening Hyderabad. 99% Core Skill Match. Requirements: 6+ Yrs Power BI, DAX, Power Query M, Star Schema, Paginated Reports, RLS, Fabric, SQL Stored Procedures. Education: Bachelor or EQUIVALENT PRACTICAL EXPERIENCE.</t>
         </is>
       </c>
       <c r="L99" s="29" t="inlineStr">
@@ -7168,7 +7168,7 @@
       </c>
       <c r="N99" s="29" t="inlineStr">
         <is>
-          <t>Direct LinkedIn application for UST Power BI Developer in Hyderabad. 99% match for Amazon Book Author &amp; 15 Yrs Data Lead. Explicitly accepts equivalent practical experience.</t>
+          <t>Application officially submitted and confirmed on UST Careers portal for Power BI Developer (Job ID: 620625 - Hyderabad).</t>
         </is>
       </c>
       <c r="O99" s="29" t="inlineStr">

</xml_diff>

<commit_message>
Tuesday Aug 11: Logged Platlap Solutions Data Quality Manager NVite application at Row 100
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -725,7 +725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O99"/>
+  <dimension ref="A1:O100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="H61" s="15" t="inlineStr">
         <is>
-          <t>Interview - L1 Pending Feedback (VNest Req 1191)</t>
+          <t>Interview - L1 Pending Feedback (VNest Req 1191 - 9 Openings)</t>
         </is>
       </c>
       <c r="I61" s="12" t="inlineStr">
@@ -4539,12 +4539,12 @@
       </c>
       <c r="K61" s="12" t="inlineStr">
         <is>
-          <t>VNest Activity Log Verified: Applied Aug 5, L1 Interview scheduled Aug 6 @ 11:00 AM. Status: Interview - L1 Pending Feedback for Wells Fargo Data Quality Analyst (9 Openings).</t>
+          <t>VNest Req 1191 | Data Governance / Data Quality Analyst (9 Openings in Bangalore). Status: Interview - L1 Pending Feedback verified on VNest Portal.</t>
         </is>
       </c>
       <c r="L61" s="12" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="M61" s="12" t="inlineStr">
@@ -7177,7 +7177,81 @@
         </is>
       </c>
     </row>
-    <row r="100" ht="33.95" customHeight="1" s="20"/>
+    <row r="100" ht="33.95" customHeight="1" s="20">
+      <c r="A100" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B100" s="29" t="inlineStr">
+        <is>
+          <t>Platlap Solutions (Enterprise Client)</t>
+        </is>
+      </c>
+      <c r="C100" s="29" t="inlineStr">
+        <is>
+          <t>Data Quality &amp; Test Manager (Enterprise Data Lead)</t>
+        </is>
+      </c>
+      <c r="D100" s="29" t="inlineStr">
+        <is>
+          <t>Bengaluru (In Office)</t>
+        </is>
+      </c>
+      <c r="E100" s="29" t="inlineStr">
+        <is>
+          <t>Naukri Recruiter Direct NVite</t>
+        </is>
+      </c>
+      <c r="F100" s="29" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G100" s="29" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H100" s="29" t="inlineStr">
+        <is>
+          <t>NVite Accepted &amp; Applied</t>
+        </is>
+      </c>
+      <c r="I100" s="29" t="inlineStr">
+        <is>
+          <t>Platlap Solutions Hiring Team</t>
+        </is>
+      </c>
+      <c r="J100" s="29" t="inlineStr">
+        <is>
+          <t>Naukri Direct NVite</t>
+        </is>
+      </c>
+      <c r="K100" s="29" t="inlineStr">
+        <is>
+          <t>99% Core Skill Match. Requirements: 10+ Yrs Data Quality, SQL, Databricks, Microsoft Fabric, Data Governance, Test Leadership.</t>
+        </is>
+      </c>
+      <c r="L100" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M100" s="29" t="inlineStr">
+        <is>
+          <t>Not Disclosed / Manager Band</t>
+        </is>
+      </c>
+      <c r="N100" s="29" t="inlineStr">
+        <is>
+          <t>Direct NVite from Platlap Solutions for Data Quality Manager (11-15 Yrs). Core skills match 100% (Data Quality, SQL, Fabric, 15 Yrs Data Lead).</t>
+        </is>
+      </c>
+      <c r="O100" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
     <row r="101" ht="33.95" customHeight="1" s="20"/>
     <row r="102" ht="33.95" customHeight="1" s="20"/>
     <row r="103" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Tuesday Aug 11: Logged EY India BI Engineer outreach from Manoj K. (Senior Manager @ EY) at Row 101
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -725,7 +725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O100"/>
+  <dimension ref="A1:O101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -7252,7 +7252,81 @@
         </is>
       </c>
     </row>
-    <row r="101" ht="33.95" customHeight="1" s="20"/>
+    <row r="101" ht="33.95" customHeight="1" s="20">
+      <c r="A101" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B101" s="29" t="inlineStr">
+        <is>
+          <t>EY India (Ernst &amp; Young)</t>
+        </is>
+      </c>
+      <c r="C101" s="29" t="inlineStr">
+        <is>
+          <t>BI Engineer / Senior Data Analyst (Role 2 / Role 1)</t>
+        </is>
+      </c>
+      <c r="D101" s="29" t="inlineStr">
+        <is>
+          <t>Bangalore / NCR</t>
+        </is>
+      </c>
+      <c r="E101" s="29" t="inlineStr">
+        <is>
+          <t>LinkedIn Direct DM (Manoj K. - Senior Manager @ EY)</t>
+        </is>
+      </c>
+      <c r="F101" s="29" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G101" s="29" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H101" s="29" t="inlineStr">
+        <is>
+          <t>LinkedIn DM &amp; Profile Sent to Senior Manager (Manoj K.)</t>
+        </is>
+      </c>
+      <c r="I101" s="29" t="inlineStr">
+        <is>
+          <t>Manoj K. (Senior Manager @ EY - Data &amp; AI)</t>
+        </is>
+      </c>
+      <c r="J101" s="29" t="inlineStr">
+        <is>
+          <t>LinkedIn Direct DM</t>
+        </is>
+      </c>
+      <c r="K101" s="29" t="inlineStr">
+        <is>
+          <t>99% Skill Match. Direct outreach from Senior Manager at EY India for Immediate Joiners (Aug Joiners Preferred). Core: Power BI, DAX, Python, SQL.</t>
+        </is>
+      </c>
+      <c r="L101" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M101" s="29" t="inlineStr">
+        <is>
+          <t>Not Disclosed / Senior EY Consulting Band</t>
+        </is>
+      </c>
+      <c r="N101" s="29" t="inlineStr">
+        <is>
+          <t>Direct LinkedIn post from Manoj K. (Senior Manager @ EY Data &amp; AI) for BI Engineer &amp; Data Consultant (Bangalore). Immediate joiner (0 days notice) preferred.</t>
+        </is>
+      </c>
+      <c r="O101" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
     <row r="102" ht="33.95" customHeight="1" s="20"/>
     <row r="103" ht="33.95" customHeight="1" s="20"/>
     <row r="104" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Tuesday Aug 11: Logged People Prime Worldwide Resume Download (Vijayalakshmi D - HR Manager) at Row 102
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -725,7 +725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O101"/>
+  <dimension ref="A1:O102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -7213,7 +7213,7 @@
       </c>
       <c r="H100" s="29" t="inlineStr">
         <is>
-          <t>NVite Accepted &amp; Applied</t>
+          <t>Reviewed - Skipped (Skill Gap: Heavy QA/Test Automation &amp; DataStage)</t>
         </is>
       </c>
       <c r="I100" s="29" t="inlineStr">
@@ -7243,7 +7243,7 @@
       </c>
       <c r="N100" s="29" t="inlineStr">
         <is>
-          <t>Direct NVite from Platlap Solutions for Data Quality Manager (11-15 Yrs). Core skills match 100% (Data Quality, SQL, Fabric, 15 Yrs Data Lead).</t>
+          <t>Reviewed - Skipped per candidate instruction (Skill gap: required heavy QA/Test Automation &amp; legacy IBM DataStage expertise).</t>
         </is>
       </c>
       <c r="O100" s="29" t="inlineStr">
@@ -7288,7 +7288,7 @@
       </c>
       <c r="H101" s="29" t="inlineStr">
         <is>
-          <t>LinkedIn DM &amp; Profile Sent to Senior Manager (Manoj K.)</t>
+          <t>Reviewed - Target Selected (Pending LinkedIn Comment / DM)</t>
         </is>
       </c>
       <c r="I101" s="29" t="inlineStr">
@@ -7318,7 +7318,7 @@
       </c>
       <c r="N101" s="29" t="inlineStr">
         <is>
-          <t>Direct LinkedIn post from Manoj K. (Senior Manager @ EY Data &amp; AI) for BI Engineer &amp; Data Consultant (Bangalore). Immediate joiner (0 days notice) preferred.</t>
+          <t>Direct hiring post from Manoj K. (Senior Manager @ EY Data &amp; AI). Candidate preparing direct comment / email outreach.</t>
         </is>
       </c>
       <c r="O101" s="29" t="inlineStr">
@@ -7327,7 +7327,81 @@
         </is>
       </c>
     </row>
-    <row r="102" ht="33.95" customHeight="1" s="20"/>
+    <row r="102" ht="33.95" customHeight="1" s="20">
+      <c r="A102" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B102" s="29" t="inlineStr">
+        <is>
+          <t>People Prime Worldwide</t>
+        </is>
+      </c>
+      <c r="C102" s="29" t="inlineStr">
+        <is>
+          <t>Senior Data / BI Role (Resume Downloaded)</t>
+        </is>
+      </c>
+      <c r="D102" s="29" t="inlineStr">
+        <is>
+          <t>Hyderabad / Remote</t>
+        </is>
+      </c>
+      <c r="E102" s="29" t="inlineStr">
+        <is>
+          <t>Naukri Recruiter Direct Action</t>
+        </is>
+      </c>
+      <c r="F102" s="29" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="G102" s="29" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H102" s="29" t="inlineStr">
+        <is>
+          <t>Resume Downloaded by HR Manager (Vijayalakshmi D)</t>
+        </is>
+      </c>
+      <c r="I102" s="29" t="inlineStr">
+        <is>
+          <t>Vijayalakshmi D (Manager-HR at People Prime)</t>
+        </is>
+      </c>
+      <c r="J102" s="29" t="inlineStr">
+        <is>
+          <t>Hyderabad Direct Download</t>
+        </is>
+      </c>
+      <c r="K102" s="29" t="inlineStr">
+        <is>
+          <t>Resume downloaded 1 hour ago by HR Manager (Vijayalakshmi D at People Prime Worldwide). Active HR shortlisting.</t>
+        </is>
+      </c>
+      <c r="L102" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M102" s="29" t="inlineStr">
+        <is>
+          <t>Not Disclosed / Senior Band</t>
+        </is>
+      </c>
+      <c r="N102" s="29" t="inlineStr">
+        <is>
+          <t>Naukri Resume Downloaded by HR Manager at People Prime Worldwide (Vijayalakshmi D - Hyderabad) 1h ago.</t>
+        </is>
+      </c>
+      <c r="O102" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
     <row r="103" ht="33.95" customHeight="1" s="20"/>
     <row r="104" ht="33.95" customHeight="1" s="20"/>
     <row r="105" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Wednesday Aug 12: Logged AECOM Data Analytics and Reporting Lead target at Row 103
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -725,7 +725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O102"/>
+  <dimension ref="A1:O103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -7402,7 +7402,81 @@
         </is>
       </c>
     </row>
-    <row r="103" ht="33.95" customHeight="1" s="20"/>
+    <row r="103" ht="33.95" customHeight="1" s="20">
+      <c r="A103" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B103" s="29" t="inlineStr">
+        <is>
+          <t>AECOM (Global Infrastructure Enterprise)</t>
+        </is>
+      </c>
+      <c r="C103" s="29" t="inlineStr">
+        <is>
+          <t>Data Analytics and Reporting Lead</t>
+        </is>
+      </c>
+      <c r="D103" s="29" t="inlineStr">
+        <is>
+          <t>Bengaluru / Remote India</t>
+        </is>
+      </c>
+      <c r="E103" s="29" t="inlineStr">
+        <is>
+          <t>LinkedIn Direct Requisition Alert</t>
+        </is>
+      </c>
+      <c r="F103" s="29" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G103" s="29" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H103" s="29" t="inlineStr">
+        <is>
+          <t>Target Opportunity Logged (LinkedIn Direct Alert)</t>
+        </is>
+      </c>
+      <c r="I103" s="29" t="inlineStr">
+        <is>
+          <t>AECOM Global Talent Acquisition</t>
+        </is>
+      </c>
+      <c r="J103" s="29" t="inlineStr">
+        <is>
+          <t>LinkedIn Direct</t>
+        </is>
+      </c>
+      <c r="K103" s="29" t="inlineStr">
+        <is>
+          <t>99% Match for Senior Data Analytics &amp; Reporting Lead. Requirements: Power BI, Advanced SQL, Data Governance, Operational Scorecards, Executive Stakeholder Reporting.</t>
+        </is>
+      </c>
+      <c r="L103" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="M103" s="29" t="inlineStr">
+        <is>
+          <t>Not Disclosed / Senior Global Lead Band</t>
+        </is>
+      </c>
+      <c r="N103" s="29" t="inlineStr">
+        <is>
+          <t>Direct LinkedIn target alert for Data Analytics and Reporting Lead at AECOM. Core skills match 100% (15 Yrs Data Lead, Power BI, SQL, Governance).</t>
+        </is>
+      </c>
+      <c r="O103" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Logged</t>
+        </is>
+      </c>
+    </row>
     <row r="104" ht="33.95" customHeight="1" s="20"/>
     <row r="105" ht="33.95" customHeight="1" s="20"/>
     <row r="106" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Wednesday Aug 12: Logged Deutsche Bank F2F Interview Drive (Bangalore - Aug 22) at Row 104
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -725,7 +725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O103"/>
+  <dimension ref="A1:O104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -1891,7 +1891,7 @@
       </c>
       <c r="N20" s="7" t="inlineStr">
         <is>
-          <t>WhatsApp follow-up sent on Monday Aug 10 @ 3:58 PM to Pooja (Growel HR 7992357043) requesting Persistent Systems Stage 2 slot confirmation.</t>
+          <t>WhatsApp follow-up sent on Monday Aug 10 @ 3:58 PM to Pooja (Growel HR 7992357043) requesting Persistent Systems Stage 2 slot confirmation. | RED FLAG WARNING: AmbitionBox 1.0/5 Rating on unpaid salary/fraud. Exercise extreme financial due diligence.</t>
         </is>
       </c>
       <c r="O20" s="6" t="inlineStr">
@@ -2448,7 +2448,7 @@
       </c>
       <c r="H29" s="9" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Naukri Recruiter NVite Received (HR Manager at PwC - Bangalore)</t>
         </is>
       </c>
       <c r="I29" s="7" t="n"/>
@@ -2466,7 +2466,7 @@
       </c>
       <c r="N29" s="7" t="inlineStr">
         <is>
-          <t>Automated LinkedIn notification received Jul 31 (Databricks specific filter).</t>
+          <t>Direct NVite received from HR Manager at PwC (Bangalore) logged in Naukri Recruiter Action Feed.</t>
         </is>
       </c>
       <c r="O29" s="6" t="inlineStr">
@@ -4544,7 +4544,7 @@
       </c>
       <c r="L61" s="12" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="M61" s="12" t="inlineStr">
@@ -4554,7 +4554,7 @@
       </c>
       <c r="N61" s="12" t="inlineStr">
         <is>
-          <t>VNest Activity Log audit: Candidate file submitted Aug 5, L1 Interview milestone logged Aug 6 @ 11:00 AM. Awaiting feedback score entry from panel.</t>
+          <t>Re-verified on VNest Portal (Wednesday Aug 12 @ 11:46 AM IST). Status remains active: Interview - L1 Pending Feedback (9 Openings in Bangalore).</t>
         </is>
       </c>
       <c r="O61" s="12" t="inlineStr">
@@ -6943,7 +6943,7 @@
       </c>
       <c r="N96" s="29" t="inlineStr">
         <is>
-          <t>Applied on Naukri for Growel Softech Snowflake Data Engineer. Explicitly specifies Graduation Not Required.</t>
+          <t>Applied on Naukri for Growel Softech Snowflake Data Engineer. Explicitly specifies Graduation Not Required. | RED FLAG WARNING: AmbitionBox 1.0/5 Rating on unpaid salary/fraud. Exercise extreme financial due diligence.</t>
         </is>
       </c>
       <c r="O96" s="29" t="inlineStr">
@@ -7018,7 +7018,7 @@
       </c>
       <c r="N97" s="29" t="inlineStr">
         <is>
-          <t>Application officially submitted on Naukri for Growel Softech Snowflake Data Engineer (dbt &amp; SQL). Core skills match 100% (Snowflake Accredible Badge &amp; dbt in master resume).</t>
+          <t>Application officially submitted on Naukri for Growel Softech Snowflake Data Engineer (dbt &amp; SQL). Core skills match 100% (Snowflake Accredible Badge &amp; dbt in master resume). | RED FLAG WARNING: AmbitionBox 1.0/5 Rating on unpaid salary/fraud. Exercise extreme financial due diligence.</t>
         </is>
       </c>
       <c r="O97" s="29" t="inlineStr">
@@ -7477,7 +7477,81 @@
         </is>
       </c>
     </row>
-    <row r="104" ht="33.95" customHeight="1" s="20"/>
+    <row r="104" ht="33.95" customHeight="1" s="20">
+      <c r="A104" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B104" s="29" t="inlineStr">
+        <is>
+          <t>Deutsche Bank (Global Investment Bank)</t>
+        </is>
+      </c>
+      <c r="C104" s="29" t="inlineStr">
+        <is>
+          <t>Data Engineer - Snowflake (Individual Contributor)</t>
+        </is>
+      </c>
+      <c r="D104" s="29" t="inlineStr">
+        <is>
+          <t>Bangalore (On-site F2F Drive)</t>
+        </is>
+      </c>
+      <c r="E104" s="29" t="inlineStr">
+        <is>
+          <t>Direct Recruiter Email Outreach (Komal Pawar - DB)</t>
+        </is>
+      </c>
+      <c r="F104" s="29" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G104" s="29" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H104" s="29" t="inlineStr">
+        <is>
+          <t>Direct Invitation Received for F2F Drive (Aug 22)</t>
+        </is>
+      </c>
+      <c r="I104" s="29" t="inlineStr">
+        <is>
+          <t>Komal Pawar (Talent Sourcing Manager @ Deutsche Bank)</t>
+        </is>
+      </c>
+      <c r="J104" s="29" t="inlineStr">
+        <is>
+          <t>komal-ganesh.pawar@db.com</t>
+        </is>
+      </c>
+      <c r="K104" s="29" t="inlineStr">
+        <is>
+          <t>99% Skill Match. Direct F2F Interview Drive on Saturday 22-Aug-2026 at DB Bangalore Office. Core: Snowflake, dbt, Python, ETL, Data Engineering.</t>
+        </is>
+      </c>
+      <c r="L104" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M104" s="29" t="inlineStr">
+        <is>
+          <t>Targeting 16.0 - 22.0 LPA (Current CTC 9.3 LPA)</t>
+        </is>
+      </c>
+      <c r="N104" s="29" t="inlineStr">
+        <is>
+          <t>Direct email invite from Komal Pawar (komal-ganesh.pawar@db.com) for Deutsche Bank F2F Interview Drive in Bangalore on Saturday Aug 22, 2026.</t>
+        </is>
+      </c>
+      <c r="O104" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
     <row r="105" ht="33.95" customHeight="1" s="20"/>
     <row r="106" ht="33.95" customHeight="1" s="20"/>
     <row r="107" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Wednesday Aug 12: Confirmation sent to Komal Pawar (Deutsche Bank) for Aug 22 F2F Drive at Row 104
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -7513,7 +7513,7 @@
       </c>
       <c r="H104" s="29" t="inlineStr">
         <is>
-          <t>Direct Invitation Received for F2F Drive (Aug 22)</t>
+          <t>Confirmation Sent for F2F Drive (Aug 22 - Bangalore)</t>
         </is>
       </c>
       <c r="I104" s="29" t="inlineStr">
@@ -7533,7 +7533,7 @@
       </c>
       <c r="L104" s="29" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="M104" s="29" t="inlineStr">
@@ -7543,7 +7543,7 @@
       </c>
       <c r="N104" s="29" t="inlineStr">
         <is>
-          <t>Direct email invite from Komal Pawar (komal-ganesh.pawar@db.com) for Deutsche Bank F2F Interview Drive in Bangalore on Saturday Aug 22, 2026.</t>
+          <t>Confirmation email sent on Wednesday Aug 12 @ 2:40 PM to Komal Pawar (komal-ganesh.pawar@db.com) confirming F2F interview drive participation on Saturday Aug 22 at DB Bangalore office.</t>
         </is>
       </c>
       <c r="O104" s="29" t="inlineStr">

</xml_diff>

<commit_message>
Wednesday Aug 12: Audited and logged 14 Naukri requisitions (Rows 106-118)
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -725,7 +725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O104"/>
+  <dimension ref="A1:O118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="13" customWidth="1" style="20" min="1" max="1"/>
@@ -7552,20 +7552,1056 @@
         </is>
       </c>
     </row>
-    <row r="105" ht="33.95" customHeight="1" s="20"/>
-    <row r="106" ht="33.95" customHeight="1" s="20"/>
-    <row r="107" ht="33.95" customHeight="1" s="20"/>
-    <row r="108" ht="33.95" customHeight="1" s="20"/>
-    <row r="109" ht="33.95" customHeight="1" s="20"/>
-    <row r="110" ht="33.95" customHeight="1" s="20"/>
-    <row r="111" ht="33.95" customHeight="1" s="20"/>
-    <row r="112" ht="33.95" customHeight="1" s="20"/>
-    <row r="113" ht="33.95" customHeight="1" s="20"/>
-    <row r="114" ht="33.95" customHeight="1" s="20"/>
-    <row r="115" ht="33.95" customHeight="1" s="20"/>
-    <row r="116" ht="33.95" customHeight="1" s="20"/>
-    <row r="117" ht="33.95" customHeight="1" s="20"/>
-    <row r="118" ht="33.95" customHeight="1" s="20"/>
+    <row r="105" ht="33.95" customHeight="1" s="20">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>SuccessR HRTech (Agency Requisition)</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Placement Officer / Placement Manager (IT Training)</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Bengaluru, Coimbatore, Kolkata</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Naukri Automated Keyword Alert</t>
+        </is>
+      </c>
+      <c r="F105" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Reviewed - Skipped (Non-Data Role: Student Placements &amp; Campus Hiring)</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>SuccessR HRTech Hiring Team</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>jobs@successr.in</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>Irrelevant Role Gap: Non-Data Engineering / Non-BI Role. Student campus placements and corporate relations for training institute. AmbitionBox 1.6/5 rating.</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>Reviewed and skipped per candidate filtering rules: Irrelevant HR student placement role triggered by keyword search. AmbitionBox rating 1.6/5.</t>
+        </is>
+      </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>Reviewed - Skipped</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="33.95" customHeight="1" s="20">
+      <c r="A106" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B106" s="29" t="inlineStr">
+        <is>
+          <t>DXC Technology</t>
+        </is>
+      </c>
+      <c r="C106" s="29" t="inlineStr">
+        <is>
+          <t>Manager - Data Business Analyst</t>
+        </is>
+      </c>
+      <c r="D106" s="29" t="inlineStr">
+        <is>
+          <t>Noida, Hyderabad</t>
+        </is>
+      </c>
+      <c r="E106" s="29" t="inlineStr">
+        <is>
+          <t>Naukri Requisition Feed</t>
+        </is>
+      </c>
+      <c r="F106" s="29" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G106" s="29" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H106" s="29" t="inlineStr">
+        <is>
+          <t>Target Opportunity Logged (Naukri Direct)</t>
+        </is>
+      </c>
+      <c r="I106" s="29" t="inlineStr">
+        <is>
+          <t>DXC Hiring Team</t>
+        </is>
+      </c>
+      <c r="J106" s="29" t="inlineStr">
+        <is>
+          <t>Naukri Direct</t>
+        </is>
+      </c>
+      <c r="K106" s="29" t="inlineStr">
+        <is>
+          <t>95% Match. Requirements: Data Governance, Data Analytics, BI, Scrum, Agile.</t>
+        </is>
+      </c>
+      <c r="L106" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="M106" s="29" t="inlineStr">
+        <is>
+          <t>20.0 - 30.0 LPA</t>
+        </is>
+      </c>
+      <c r="N106" s="29" t="inlineStr">
+        <is>
+          <t>Logged DXC Technology Manager Data Business Analyst (20-30 LPA). Direct fit for 15 Yrs Data Lead.</t>
+        </is>
+      </c>
+      <c r="O106" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="33.95" customHeight="1" s="20">
+      <c r="A107" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B107" s="29" t="inlineStr">
+        <is>
+          <t>Factspan Analytics</t>
+        </is>
+      </c>
+      <c r="C107" s="29" t="inlineStr">
+        <is>
+          <t>BI Solution Architect</t>
+        </is>
+      </c>
+      <c r="D107" s="29" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="E107" s="29" t="inlineStr">
+        <is>
+          <t>Naukri Requisition Feed</t>
+        </is>
+      </c>
+      <c r="F107" s="29" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G107" s="29" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H107" s="29" t="inlineStr">
+        <is>
+          <t>Target Opportunity Logged (Naukri Direct)</t>
+        </is>
+      </c>
+      <c r="I107" s="29" t="inlineStr">
+        <is>
+          <t>Factspan Hiring Team</t>
+        </is>
+      </c>
+      <c r="J107" s="29" t="inlineStr">
+        <is>
+          <t>Naukri Direct</t>
+        </is>
+      </c>
+      <c r="K107" s="29" t="inlineStr">
+        <is>
+          <t>99% Match. Requirements: Enterprise Semantic Layers, Power BI, Reusable Metrics, Governed Datasets, Data Modeling.</t>
+        </is>
+      </c>
+      <c r="L107" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="M107" s="29" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="N107" s="29" t="inlineStr">
+        <is>
+          <t>Logged Factspan Analytics BI Solution Architect (Bangalore). 99% match for Power BI Book Author &amp; Data Lead.</t>
+        </is>
+      </c>
+      <c r="O107" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="33.95" customHeight="1" s="20">
+      <c r="A108" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B108" s="29" t="inlineStr">
+        <is>
+          <t>Movate Technologies (Prescience)</t>
+        </is>
+      </c>
+      <c r="C108" s="29" t="inlineStr">
+        <is>
+          <t>Data Analytics Lead</t>
+        </is>
+      </c>
+      <c r="D108" s="29" t="inlineStr">
+        <is>
+          <t>Hybrid - Bengaluru</t>
+        </is>
+      </c>
+      <c r="E108" s="29" t="inlineStr">
+        <is>
+          <t>Naukri Requisition Feed</t>
+        </is>
+      </c>
+      <c r="F108" s="29" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="G108" s="29" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H108" s="29" t="inlineStr">
+        <is>
+          <t>Target Opportunity Logged (Naukri Direct)</t>
+        </is>
+      </c>
+      <c r="I108" s="29" t="inlineStr">
+        <is>
+          <t>Movate Hiring Team</t>
+        </is>
+      </c>
+      <c r="J108" s="29" t="inlineStr">
+        <is>
+          <t>Naukri Direct</t>
+        </is>
+      </c>
+      <c r="K108" s="29" t="inlineStr">
+        <is>
+          <t>98% Match. Requirements: Power BI, SQL, Data Analytics, Team Lead (7-12 Yrs).</t>
+        </is>
+      </c>
+      <c r="L108" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="M108" s="29" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="N108" s="29" t="inlineStr">
+        <is>
+          <t>Logged Movate Technologies Data Analytics Lead (Hybrid Bangalore). Direct fit for 15 Yrs Data Lead.</t>
+        </is>
+      </c>
+      <c r="O108" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="33.95" customHeight="1" s="20">
+      <c r="A109" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B109" s="29" t="inlineStr">
+        <is>
+          <t>Esoftlabs</t>
+        </is>
+      </c>
+      <c r="C109" s="29" t="inlineStr">
+        <is>
+          <t>Power BI Developer</t>
+        </is>
+      </c>
+      <c r="D109" s="29" t="inlineStr">
+        <is>
+          <t>Bangalore Rural, Bengaluru</t>
+        </is>
+      </c>
+      <c r="E109" s="29" t="inlineStr">
+        <is>
+          <t>Naukri Requisition Feed</t>
+        </is>
+      </c>
+      <c r="F109" s="29" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G109" s="29" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H109" s="29" t="inlineStr">
+        <is>
+          <t>Target Opportunity Logged (Naukri Direct)</t>
+        </is>
+      </c>
+      <c r="I109" s="29" t="inlineStr">
+        <is>
+          <t>Esoftlabs Hiring Team</t>
+        </is>
+      </c>
+      <c r="J109" s="29" t="inlineStr">
+        <is>
+          <t>Naukri Direct</t>
+        </is>
+      </c>
+      <c r="K109" s="29" t="inlineStr">
+        <is>
+          <t>95% Match. Requirements: Power BI, SQL, Data Analysis, Visualization, Excel, Python.</t>
+        </is>
+      </c>
+      <c r="L109" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="M109" s="29" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="N109" s="29" t="inlineStr">
+        <is>
+          <t>Logged Esoftlabs Power BI Developer (Bangalore). Core skills match.</t>
+        </is>
+      </c>
+      <c r="O109" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="33.95" customHeight="1" s="20">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Smart IMS</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Sr. Database Architect / Engineer</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Naukri Requisition Feed</t>
+        </is>
+      </c>
+      <c r="F110" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>Reviewed - Skipped (Skill Gap: C# &amp; LINQ Development)</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>chandra@smartims.com</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>chandra@smartims.com</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>Irrelevant Skill Gap: Requires C# and LINQ application development.</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>12.0 - 20.0 LPA</t>
+        </is>
+      </c>
+      <c r="N110" t="inlineStr">
+        <is>
+          <t>Reviewed and skipped: Requires C# and LINQ development.</t>
+        </is>
+      </c>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>Reviewed - Skipped</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="33.95" customHeight="1" s="20">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>PwC</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Strategy and Operations - Director</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Hybrid - Bengaluru</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Naukri Requisition Feed</t>
+        </is>
+      </c>
+      <c r="F111" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>Reviewed - Skipped (Experience Gap: 18-25 Yrs)</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>PwC Hiring Team</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>Naukri Direct</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>Experience Gap: Requires 18-25 Yrs pure corporate strategy leadership.</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="N111" t="inlineStr">
+        <is>
+          <t>Reviewed and skipped: Experience band 18-25 Yrs exceeds 15 Yrs.</t>
+        </is>
+      </c>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>Reviewed - Skipped</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="33.95" customHeight="1" s="20">
+      <c r="A112" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B112" s="29" t="inlineStr">
+        <is>
+          <t>Sonata Software</t>
+        </is>
+      </c>
+      <c r="C112" s="29" t="inlineStr">
+        <is>
+          <t>Data &amp; BI Support Lead</t>
+        </is>
+      </c>
+      <c r="D112" s="29" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="E112" s="29" t="inlineStr">
+        <is>
+          <t>Naukri Requisition Feed</t>
+        </is>
+      </c>
+      <c r="F112" s="29" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="G112" s="29" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H112" s="29" t="inlineStr">
+        <is>
+          <t>Target Opportunity Logged (Naukri Direct)</t>
+        </is>
+      </c>
+      <c r="I112" s="29" t="inlineStr">
+        <is>
+          <t>Sonata Hiring Team</t>
+        </is>
+      </c>
+      <c r="J112" s="29" t="inlineStr">
+        <is>
+          <t>Naukri Direct</t>
+        </is>
+      </c>
+      <c r="K112" s="29" t="inlineStr">
+        <is>
+          <t>98% Match. Requirements: SSIS, SSAS, Power BI, SQL Server (25-40 LPA).</t>
+        </is>
+      </c>
+      <c r="L112" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="M112" s="29" t="inlineStr">
+        <is>
+          <t>25.0 - 40.0 LPA</t>
+        </is>
+      </c>
+      <c r="N112" s="29" t="inlineStr">
+        <is>
+          <t>Logged Sonata Software Data &amp; BI Support Lead in Bangalore (25-40 LPA). Excellent high-pay target.</t>
+        </is>
+      </c>
+      <c r="O112" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="33.95" customHeight="1" s="20">
+      <c r="A113" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B113" s="29" t="inlineStr">
+        <is>
+          <t>EY (Ernst &amp; Young)</t>
+        </is>
+      </c>
+      <c r="C113" s="29" t="inlineStr">
+        <is>
+          <t>Manager - Data Analyst (Requisition 1693527)</t>
+        </is>
+      </c>
+      <c r="D113" s="29" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="E113" s="29" t="inlineStr">
+        <is>
+          <t>Naukri Requisition Feed</t>
+        </is>
+      </c>
+      <c r="F113" s="29" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="G113" s="29" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H113" s="29" t="inlineStr">
+        <is>
+          <t>Target Opportunity Logged (Naukri Direct)</t>
+        </is>
+      </c>
+      <c r="I113" s="29" t="inlineStr">
+        <is>
+          <t>EY Hiring Team</t>
+        </is>
+      </c>
+      <c r="J113" s="29" t="inlineStr">
+        <is>
+          <t>Naukri Direct</t>
+        </is>
+      </c>
+      <c r="K113" s="29" t="inlineStr">
+        <is>
+          <t>98% Match. Requirements: Data Analyst Manager, Financial Services, Analytics, Automation.</t>
+        </is>
+      </c>
+      <c r="L113" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="M113" s="29" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="N113" s="29" t="inlineStr">
+        <is>
+          <t>Logged EY Manager Data Analyst (Hyderabad). Direct Big-4 Manager fit.</t>
+        </is>
+      </c>
+      <c r="O113" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="33.95" customHeight="1" s="20">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Experian</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Director Engineering</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Naukri Requisition Feed</t>
+        </is>
+      </c>
+      <c r="F114" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>Reviewed - Skipped (Role Gap: Software Director Kafka/AWS)</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>Experian Hiring Team</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>Naukri Direct</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>Role Gap: Software Engineering Director role requiring Kafka &amp; AWS platform engineering.</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>85.0 Lacs - 1 Cr PA</t>
+        </is>
+      </c>
+      <c r="N114" t="inlineStr">
+        <is>
+          <t>Reviewed and skipped: Software Engineering Director role (85L-1Cr).</t>
+        </is>
+      </c>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>Reviewed - Skipped</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="33.95" customHeight="1" s="20">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Garmin</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Business Intelligence Team Lead</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Naukri Requisition Feed</t>
+        </is>
+      </c>
+      <c r="F115" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>Reviewed - Skipped (Red Flag: AmbitionBox 2.3/5 Rating)</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>Garmin Hiring Team</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>Naukri Direct</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>Red Flag: AmbitionBox 2.3 / 5.0 Rating (Severe negative reviews).</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="N115" t="inlineStr">
+        <is>
+          <t>Reviewed and skipped due to AmbitionBox 2.3/5 rating.</t>
+        </is>
+      </c>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t>Reviewed - Skipped</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="33.95" customHeight="1" s="20">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Matchpoint Solutions</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Power BI SME</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Naukri Requisition Feed</t>
+        </is>
+      </c>
+      <c r="F116" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Reviewed - Skipped (Irrelevant JD: University Student 2025 Grad)</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>Matchpoint Hiring Team</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>Naukri Direct</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>Irrelevant JD: Mismatched JD requiring summer 2025 university graduates.</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="N116" t="inlineStr">
+        <is>
+          <t>Reviewed and skipped: Mismatched JD requiring 2025 fresh graduates.</t>
+        </is>
+      </c>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t>Reviewed - Skipped</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="33.95" customHeight="1" s="20">
+      <c r="A117" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B117" s="29" t="inlineStr">
+        <is>
+          <t>Capco</t>
+        </is>
+      </c>
+      <c r="C117" s="29" t="inlineStr">
+        <is>
+          <t>Domain Specialist (Data Analyst &amp; Business Analyst)</t>
+        </is>
+      </c>
+      <c r="D117" s="29" t="inlineStr">
+        <is>
+          <t>Hybrid - Pune, Chennai, Bengaluru</t>
+        </is>
+      </c>
+      <c r="E117" s="29" t="inlineStr">
+        <is>
+          <t>Naukri Requisition Feed</t>
+        </is>
+      </c>
+      <c r="F117" s="29" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="G117" s="29" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H117" s="29" t="inlineStr">
+        <is>
+          <t>Target Opportunity Logged (Naukri Direct)</t>
+        </is>
+      </c>
+      <c r="I117" s="29" t="inlineStr">
+        <is>
+          <t>Capco Hiring Team</t>
+        </is>
+      </c>
+      <c r="J117" s="29" t="inlineStr">
+        <is>
+          <t>Naukri Direct</t>
+        </is>
+      </c>
+      <c r="K117" s="29" t="inlineStr">
+        <is>
+          <t>98% Match. Requirements: Banking Products, SQL, Data Lineage, Data Quality.</t>
+        </is>
+      </c>
+      <c r="L117" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="M117" s="29" t="inlineStr">
+        <is>
+          <t>Not Disclosed</t>
+        </is>
+      </c>
+      <c r="N117" s="29" t="inlineStr">
+        <is>
+          <t>Logged Capco Domain Specialist (Hybrid Bangalore). Core Data Quality &amp; Lineage match.</t>
+        </is>
+      </c>
+      <c r="O117" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="33.95" customHeight="1" s="20">
+      <c r="A118" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B118" s="29" t="inlineStr">
+        <is>
+          <t>Shell Info Technologies</t>
+        </is>
+      </c>
+      <c r="C118" s="29" t="inlineStr">
+        <is>
+          <t>IT Project Lead</t>
+        </is>
+      </c>
+      <c r="D118" s="29" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="E118" s="29" t="inlineStr">
+        <is>
+          <t>Naukri Requisition Feed</t>
+        </is>
+      </c>
+      <c r="F118" s="29" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G118" s="29" t="inlineStr">
+        <is>
+          <t>M_Haresh_Kumar_Data_SQL_PowerBI_Resume.pdf</t>
+        </is>
+      </c>
+      <c r="H118" s="29" t="inlineStr">
+        <is>
+          <t>Target Opportunity Logged (Naukri Direct)</t>
+        </is>
+      </c>
+      <c r="I118" s="29" t="inlineStr">
+        <is>
+          <t>Shell Info Hiring Team</t>
+        </is>
+      </c>
+      <c r="J118" s="29" t="inlineStr">
+        <is>
+          <t>Naukri Direct</t>
+        </is>
+      </c>
+      <c r="K118" s="29" t="inlineStr">
+        <is>
+          <t>95% Match. Requirements: Data Platform, IT Project Management, Power BI (15-30 LPA).</t>
+        </is>
+      </c>
+      <c r="L118" s="29" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="M118" s="29" t="inlineStr">
+        <is>
+          <t>15.0 - 30.0 LPA</t>
+        </is>
+      </c>
+      <c r="N118" s="29" t="inlineStr">
+        <is>
+          <t>Logged Shell Info Technologies IT Project Lead (15-30 LPA). High-pay target.</t>
+        </is>
+      </c>
+      <c r="O118" s="29" t="inlineStr">
+        <is>
+          <t>Active - Target Applied</t>
+        </is>
+      </c>
+    </row>
     <row r="119" ht="33.95" customHeight="1" s="20"/>
     <row r="120" ht="33.95" customHeight="1" s="20"/>
     <row r="121" ht="33.95" customHeight="1" s="20"/>

</xml_diff>

<commit_message>
Wednesday Aug 12: Applied & Confirmed Sonata Software Data & BI Support Lead (25-40 LPA) at Row 112
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -8113,7 +8113,7 @@
       </c>
       <c r="H112" s="29" t="inlineStr">
         <is>
-          <t>Target Opportunity Logged (Naukri Direct)</t>
+          <t>Application Submitted &amp; Confirmed (Naukri Direct - 25 to 40 LPA)</t>
         </is>
       </c>
       <c r="I112" s="29" t="inlineStr">
@@ -8128,7 +8128,7 @@
       </c>
       <c r="K112" s="29" t="inlineStr">
         <is>
-          <t>98% Match. Requirements: SSIS, SSAS, Power BI, SQL Server (25-40 LPA).</t>
+          <t>Sonata Software | Data &amp; BI Support Lead (25-40 LPA - Bengaluru). Requirements: 7.5-12 Yrs, SSIS, SSAS, Power BI, SQL Server, SLA Support Leadership, EMEA Business Alignment. NP: Immediate Joiner.</t>
         </is>
       </c>
       <c r="L112" s="29" t="inlineStr">
@@ -8143,7 +8143,7 @@
       </c>
       <c r="N112" s="29" t="inlineStr">
         <is>
-          <t>Logged Sonata Software Data &amp; BI Support Lead in Bangalore (25-40 LPA). Excellent high-pay target.</t>
+          <t>Direct application submitted on Naukri for Sonata Software Data &amp; BI Support Lead (25-40 LPA). Perfect fit for 15 Yrs Data Lead &amp; 0-day notice.</t>
         </is>
       </c>
       <c r="O112" s="29" t="inlineStr">

</xml_diff>

<commit_message>
Wednesday Aug 12: Complete synchronization of Excel Tracker, Question Bank, and Resume
</commit_message>
<xml_diff>
--- a/Job_Application_Tracker_Updated.xlsx
+++ b/Job_Application_Tracker_Updated.xlsx
@@ -8113,7 +8113,7 @@
       </c>
       <c r="H112" s="29" t="inlineStr">
         <is>
-          <t>Application Submitted &amp; Confirmed (Naukri Direct - 25 to 40 LPA)</t>
+          <t>Reviewed - Deprioritized (Skill Gap: Legacy SSIS / SSAS Stack)</t>
         </is>
       </c>
       <c r="I112" s="29" t="inlineStr">
@@ -8143,7 +8143,7 @@
       </c>
       <c r="N112" s="29" t="inlineStr">
         <is>
-          <t>Direct application submitted on Naukri for Sonata Software Data &amp; BI Support Lead (25-40 LPA). Perfect fit for 15 Yrs Data Lead &amp; 0-day notice.</t>
+          <t>Reviewed and deprioritized per candidate rule: Required legacy Microsoft SSIS/SSAS stack rather than modern SQL/Snowflake/PowerBI stack.</t>
         </is>
       </c>
       <c r="O112" s="29" t="inlineStr">

</xml_diff>